<commit_message>
[Track-619] update project notification template and actions
</commit_message>
<xml_diff>
--- a/epictrack-api/src/api/templates/event_templates/project_notification/003_Project_Notification.xlsx
+++ b/epictrack-api/src/api/templates/event_templates/project_notification/003_Project_Notification.xlsx
@@ -16,9 +16,6 @@
     <sheet name="Outcome_Temp" sheetId="6" state="visible" r:id="rId7"/>
     <sheet name="Action_Temp" sheetId="7" state="visible" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Events!$A$1:$M$62</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Outcomes!$A$1:$F$15</definedName>
@@ -33,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="232">
   <si>
     <t xml:space="preserve">No</t>
   </si>
@@ -444,7 +441,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Decision: Project Notification", "new_name": "Decision: Project Notification" }</t>
+    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Decision: Project Notification", "new_name": "Decision: Project Notification","use_phase_start":"True" }</t>
   </si>
   <si>
     <r>
@@ -499,7 +496,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Notification Decision Announcement &amp; Tweet", "new_name": "Notification Decision Announcement &amp; Tweet" }</t>
+    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Notification Decision Announcement &amp; Tweet", "new_name": "Notification Decision Announcement &amp; Tweet", "use_phase_start":"True" }</t>
   </si>
   <si>
     <r>
@@ -554,42 +551,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Executive Calendar Notification", "new_name": "Executive Calendar Notification" }</t>
+    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Executive Calendar Notification", "new_name": "Executive Calendar Notification","use_phase_start":"True" }</t>
   </si>
   <si>
     <t xml:space="preserve">SetEventsStatus</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Set “Notification Review | </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Project Notification Report referred to Decision Maker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">” to INACTIVE</t>
-    </r>
+    <t xml:space="preserve">Set "Notification Review | Project Notification Report referred to Decision Maker" to INACTIVE</t>
   </si>
   <si>
     <t xml:space="preserve">[{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Report referred to Decision Maker", "is_active": false }]</t>
@@ -598,7 +566,7 @@
     <t xml:space="preserve">SetPhasesStatus</t>
   </si>
   <si>
-    <t xml:space="preserve">Set finalPhase “Notification Decision” to INACTIVE</t>
+    <t xml:space="preserve">Set finalPhase "Notification Decision" to INACTIVE</t>
   </si>
   <si>
     <t xml:space="preserve">[{"phase_name":"Notification Decision","work_type_id": 1, "ea_act_id": 3, "is_active": false }]</t>
@@ -658,6 +626,18 @@
     <t xml:space="preserve">{"start_date_locked": true}</t>
   </si>
   <si>
+    <t xml:space="preserve">{"work_type_id": 1, "ea_act_id": 3, "event_name": "Decision: Project Notification", "new_name": "Decision: Project Notification", "use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"work_type_id": 1, "ea_act_id": 3, "event_name": "Notification Decision Announcement &amp; Tweet", "new_name": "Notification Decision Announcement &amp; Tweet","use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"work_type_id": 1, "ea_act_id": 3, "event_name": "Executive Calendar Notification", "new_name": "Executive Calendar Notification","use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Report referred to Decision Maker", "is_active": false }]</t>
+  </si>
+  <si>
     <t xml:space="preserve">Set workState to TERMINATED</t>
   </si>
   <si>
@@ -688,59 +668,13 @@
     <t xml:space="preserve">SetEventName</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Rename </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">"Start of Intake Phase (e.g. Initial Contact, Draft Sharing, or PN Submission)" to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"Start of Revised PN Development"</t>
-    </r>
+    <t xml:space="preserve">Rename "Start of Intake Phase (e.g. Initial Contact, Draft Sharing, or PN Submission)" to "Start of Revised PN Development"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Project Notification Development","work_type_id": 1, "ea_act_id": 3, "event_name": "Start of Intake Phase (e.g. Initial Contact, Draft Sharing, or PN Submission)", "new_name": "Start of Revised PN Development" }</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Rename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> "Last Day of Intake Phase (day before formal submission)" to "Last Day of Revised PN Development Phase (day before re-submission)"</t>
-    </r>
+    <t xml:space="preserve">Rename "Last Day of Intake Phase (day before formal submission)" to "Last Day of Revised PN Development Phase (day before re-submission)"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Project Notification Development","work_type_id": 1, "ea_act_id": 3, "event_name": "Last Day of Intake Phase (day before formal submission)", "new_name": "Last Day of Revised PN Development Phase (day before re-submission)" }</t>
@@ -752,49 +686,13 @@
     <t xml:space="preserve">[{"phase_name":"Revised Project Notification Development","work_type_id": 1, "ea_act_id": 3, "event_name": "Meeting with Proponent", "is_active": false }]</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Rename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> "Project Notification Submission Received (Day Zero)" to "Revised PN Submission Received"</t>
-    </r>
+    <t xml:space="preserve">Rename "Project Notification Submission Received (Day Zero)" to "Revised PN Submission Received"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Submission Received (Day Zero)", "new_name": "Revised PN Submission Received" }</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Rename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> "Project Notification Report referred to Decision Maker" to "Revised PN Report referred to Decision Maker"</t>
-    </r>
+    <t xml:space="preserve">Rename "Project Notification Report referred to Decision Maker" to "Revised PN Report referred to Decision Maker"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Report referred to Decision Maker", "new_name": "Revised PN Report referred to Decision Maker" } </t>
@@ -809,13 +707,16 @@
     <t xml:space="preserve">AddEvent "Revised Notification Review | Comment Period" and set visibility to SUGGESTED (copy of Comment Period)</t>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Comment Period","visibility": "SUGGESTED" }</t>
+    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Comment Period","visibility": "SUGGESTED", "start_at": "14", "use_phase_start":"True" }</t>
   </si>
   <si>
     <t xml:space="preserve">AddEvent "Revised Notification Review | Delegation of PN Decision" and set visibility to SUGGESTED (renamed copy of Delegation of Decision)</t>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Delegation of PN Decision", "new_name": "Delegation of PN Decision","visibility": "SUGGESTED", "start_at": 1 }</t>
+    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Delegation of PN Decision", "new_name": "Delegation of PN Decision","visibility": "SUGGESTED", "start_at": "7", "use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Comment Period","visibility": "SUGGESTED", "start_at": "14", "use_phase_start":"True"}</t>
   </si>
   <si>
     <t xml:space="preserve">EA Act</t>
@@ -982,7 +883,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1040,12 +941,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1156,7 +1051,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1261,10 +1156,6 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1290,7 +1181,92 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="15">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCCCCC"/>
+          <bgColor rgb="FF272727"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2E75B6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCCCFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF3F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFBE5D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="1"/>
@@ -1312,6 +1288,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2F75B5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1387,305 +1370,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Phases"/>
-      <sheetName val="Events"/>
-      <sheetName val="Outcomes"/>
-      <sheetName val="Actions"/>
-      <sheetName val="Lookups"/>
-      <sheetName val="Outcome_Temp"/>
-      <sheetName val="Action_Temp"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2">
-        <row r="2">
-          <cell r="A2">
-            <v>1</v>
-          </cell>
-          <cell r="B2">
-            <v>6</v>
-          </cell>
-          <cell r="C2" t="str">
-            <v>EAO's Viewpoint on Submitted Document</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>Viewpoint is POSITIVE</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>2</v>
-          </cell>
-          <cell r="B3">
-            <v>6</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>EAO's Viewpoint on Submitted Document</v>
-          </cell>
-          <cell r="D3" t="str">
-            <v>Viewpoint is NEGATIVE</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>3</v>
-          </cell>
-          <cell r="B4">
-            <v>7</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>Minister's Decision</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>4</v>
-          </cell>
-          <cell r="B5">
-            <v>7</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>CEAO's Decision</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>5</v>
-          </cell>
-          <cell r="B6">
-            <v>8</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>Project Notification Withdrawn</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>PN Submission Withdrawn</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>6</v>
-          </cell>
-          <cell r="B7">
-            <v>9</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>Direct Submission of Project Notification - DELETE this Intake Phase!</v>
-          </cell>
-          <cell r="D7" t="str">
-            <v>Delete the Intake Phase</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>7</v>
-          </cell>
-          <cell r="B8">
-            <v>12</v>
-          </cell>
-          <cell r="C8" t="str">
-            <v>Project Notification Submission Received (Day Zero)</v>
-          </cell>
-          <cell r="D8" t="str">
-            <v>Start the Review Period</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>8</v>
-          </cell>
-          <cell r="B9">
-            <v>14</v>
-          </cell>
-          <cell r="C9" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D9" t="str">
-            <v>Minister's Decision</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>9</v>
-          </cell>
-          <cell r="B10">
-            <v>14</v>
-          </cell>
-          <cell r="C10" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D10" t="str">
-            <v>CEAO's Decision</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>10</v>
-          </cell>
-          <cell r="B11">
-            <v>36</v>
-          </cell>
-          <cell r="C11" t="str">
-            <v>Project Notification Terminated s.39(d)</v>
-          </cell>
-          <cell r="D11" t="str">
-            <v>PN is Terminated (s.39)</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>11</v>
-          </cell>
-          <cell r="B12">
-            <v>39</v>
-          </cell>
-          <cell r="C12" t="str">
-            <v>Project Notification Withdrawn</v>
-          </cell>
-          <cell r="D12" t="str">
-            <v>PN Submission Withdrawn</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>12</v>
-          </cell>
-          <cell r="B13">
-            <v>44</v>
-          </cell>
-          <cell r="C13" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D13" t="str">
-            <v>No Further Review Required</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>13</v>
-          </cell>
-          <cell r="B14">
-            <v>44</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D14" t="str">
-            <v>Revised PN Submission Required</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>14</v>
-          </cell>
-          <cell r="B15">
-            <v>44</v>
-          </cell>
-          <cell r="C15" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D15" t="str">
-            <v>Referred for Minister's Designation</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>15</v>
-          </cell>
-          <cell r="B16">
-            <v>52</v>
-          </cell>
-          <cell r="C16" t="str">
-            <v>Project Notification Terminated s.39(d)</v>
-          </cell>
-          <cell r="D16" t="str">
-            <v>PN is Terminated (s.39)</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>16</v>
-          </cell>
-          <cell r="B17">
-            <v>55</v>
-          </cell>
-          <cell r="C17" t="str">
-            <v>Project Notification Withdrawn</v>
-          </cell>
-          <cell r="D17" t="str">
-            <v>PN Submission Withdrawn</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18">
-            <v>17</v>
-          </cell>
-          <cell r="B18">
-            <v>59</v>
-          </cell>
-          <cell r="C18" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D18" t="str">
-            <v>No Further Review Required</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19">
-            <v>18</v>
-          </cell>
-          <cell r="B19">
-            <v>59</v>
-          </cell>
-          <cell r="C19" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D19" t="str">
-            <v>Revised PN Submission Required</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20">
-            <v>19</v>
-          </cell>
-          <cell r="B20">
-            <v>59</v>
-          </cell>
-          <cell r="C20" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D20" t="str">
-            <v>Referred for Minister's Designation</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="50.67"/>
@@ -1693,7 +1384,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="14.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="2" width="12.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="10.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1769,7 +1460,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F3" s="6" t="n">
         <f aca="false">TRUE()</f>
@@ -1817,22 +1508,22 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C4" type="list">
       <formula1>Lookups!$B$3:$B$16</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D2:D4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D2:D4" type="list">
       <formula1>Lookups!$D$3:$D$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F4" type="list">
       <formula1>Lookups!$F$3:$F$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1846,21 +1537,21 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M62"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="51.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="17.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="51.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="17.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="13.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="14.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="9.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="3.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="11.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="3.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="11.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="2" width="14.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="10.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="14" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="14" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2178,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K8" s="1" t="n">
         <v>0</v>
@@ -2587,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1" t="n">
         <v>0</v>
@@ -2922,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K26" s="1" t="n">
         <v>0</v>
@@ -3644,7 +3335,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
@@ -3672,7 +3363,7 @@
         <v>0</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K44" s="1" t="n">
         <v>0</v>
@@ -3684,7 +3375,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="n">
         <v>44</v>
       </c>
@@ -3712,7 +3403,7 @@
         <v>0</v>
       </c>
       <c r="J45" s="21" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K45" s="1" t="n">
         <v>0</v>
@@ -4437,46 +4128,46 @@
   </sheetData>
   <autoFilter ref="A1:M62"/>
   <conditionalFormatting sqref="H1:H62">
-    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="END" dxfId="0">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="END" dxfId="12">
       <formula>NOT(ISERROR(SEARCH("END",H1)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="START" dxfId="1">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="START" dxfId="13">
       <formula>NOT(ISERROR(SEARCH("START",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F62" type="list">
       <formula1>Lookups!$I$3:$I$39</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I62" type="list">
       <formula1>Lookups!$S$3:$S$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G62" type="list">
       <formula1>Lookups!$K$3:$K$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C62" type="list">
       <formula1>Phases!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L2:L3 L5:L62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L2:L3 L5:L62" type="list">
       <formula1>Lookups!$M$3:$M$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H2:H62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H2:H62" type="list">
       <formula1>Lookups!$Q$3:$Q$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L4" type="list">
       <formula1>Lookups!$M$3:$M$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4491,15 +4182,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F72"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="6.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="30.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="70.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="70.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="7" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="7" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5559,14 +5250,14 @@
   </sheetData>
   <autoFilter ref="A1:F15"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B57" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B57" type="list">
       <formula1>Events!$A$2:$A$62</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5581,16 +5272,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="7.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="18.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="116.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="63.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="87.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5736,7 +5427,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
@@ -5760,7 +5451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
@@ -6042,7 +5733,7 @@
         <v>119</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>18</v>
@@ -6066,7 +5757,7 @@
         <v>121</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>19</v>
@@ -6090,13 +5781,13 @@
         <v>123</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
@@ -6114,13 +5805,13 @@
         <v>126</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
@@ -6231,10 +5922,10 @@
         <v>135</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G27" s="1" t="n">
         <v>26</v>
@@ -6375,10 +6066,10 @@
         <v>135</v>
       </c>
       <c r="E33" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G33" s="1" t="n">
         <v>32</v>
@@ -6408,7 +6099,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
         <v>34</v>
       </c>
@@ -6420,13 +6111,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F35" s="21" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G35" s="1" t="n">
         <v>34</v>
@@ -6440,23 +6131,23 @@
         <v>13</v>
       </c>
       <c r="C36" s="9" t="str">
-        <f aca="false">IF((B36=""),"",VLOOKUP(B36,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B36=""),"",VLOOKUP(B36,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D36" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E36" s="25" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F36" s="21" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="G36" s="1" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
@@ -6468,19 +6159,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G37" s="1" t="n">
         <v>36</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="n">
         <v>37</v>
       </c>
@@ -6492,13 +6183,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E38" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
+      </c>
+      <c r="E38" s="25" t="s">
+        <v>165</v>
       </c>
       <c r="F38" s="21" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G38" s="1" t="n">
         <v>37</v>
@@ -6519,16 +6210,16 @@
         <v>125</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F39" s="21" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G39" s="1" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
@@ -6540,19 +6231,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E40" s="26" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="F40" s="21" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="G40" s="1" t="n">
         <v>39</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="n">
         <v>40</v>
       </c>
@@ -6564,13 +6255,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E41" s="26" t="s">
-        <v>167</v>
+        <v>162</v>
+      </c>
+      <c r="E41" s="25" t="s">
+        <v>171</v>
       </c>
       <c r="F41" s="21" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G41" s="1" t="n">
         <v>40</v>
@@ -6584,17 +6275,17 @@
         <v>13</v>
       </c>
       <c r="C42" s="9" t="str">
-        <f aca="false">IF((B42=""),"",VLOOKUP(B42,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B42=""),"",VLOOKUP(B42,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E42" s="25" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F42" s="21" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="G42" s="1" t="n">
         <v>41</v>
@@ -6608,17 +6299,17 @@
         <v>13</v>
       </c>
       <c r="C43" s="9" t="str">
-        <f aca="false">IF((B43=""),"",VLOOKUP(B43,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B43=""),"",VLOOKUP(B43,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D43" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="F43" s="21" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="G43" s="1" t="n">
         <v>42</v>
@@ -6632,17 +6323,17 @@
         <v>13</v>
       </c>
       <c r="C44" s="9" t="str">
-        <f aca="false">IF((B44=""),"",VLOOKUP(B44,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B44=""),"",VLOOKUP(B44,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D44" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E44" s="25" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F44" s="21" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G44" s="1" t="n">
         <v>43</v>
@@ -6663,10 +6354,10 @@
         <v>135</v>
       </c>
       <c r="E45" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G45" s="1" t="n">
         <v>44</v>
@@ -6735,10 +6426,10 @@
         <v>135</v>
       </c>
       <c r="E48" s="25" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F48" s="21" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G48" s="1" t="n">
         <v>47</v>
@@ -6879,10 +6570,10 @@
         <v>135</v>
       </c>
       <c r="E54" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G54" s="1" t="n">
         <v>53</v>
@@ -6912,7 +6603,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="n">
         <v>55</v>
       </c>
@@ -6924,13 +6615,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E56" s="25" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F56" s="21" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G56" s="1" t="n">
         <v>55</v>
@@ -6941,26 +6632,26 @@
         <v>56</v>
       </c>
       <c r="B57" s="12" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C57" s="9" t="str">
-        <f aca="false">IF((B57=""),"",VLOOKUP(B57,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B57=""),"",VLOOKUP(B57,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D57" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E57" s="25" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F57" s="21" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="G57" s="1" t="n">
         <v>56</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="n">
         <v>57</v>
       </c>
@@ -6972,19 +6663,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E58" s="25" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G58" s="1" t="n">
         <v>57</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="n">
         <v>58</v>
       </c>
@@ -6996,13 +6687,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E59" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
+      </c>
+      <c r="E59" s="25" t="s">
+        <v>165</v>
       </c>
       <c r="F59" s="21" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G59" s="1" t="n">
         <v>58</v>
@@ -7023,16 +6714,16 @@
         <v>125</v>
       </c>
       <c r="E60" s="25" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F60" s="21" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G60" s="1" t="n">
         <v>59</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="n">
         <v>60</v>
       </c>
@@ -7044,19 +6735,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E61" s="26" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="E61" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="F61" s="21" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="G61" s="1" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="n">
         <v>61</v>
       </c>
@@ -7068,13 +6759,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E62" s="26" t="s">
-        <v>167</v>
+        <v>162</v>
+      </c>
+      <c r="E62" s="25" t="s">
+        <v>171</v>
       </c>
       <c r="F62" s="21" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G62" s="1" t="n">
         <v>61</v>
@@ -7088,17 +6779,17 @@
         <v>18</v>
       </c>
       <c r="C63" s="9" t="str">
-        <f aca="false">IF((B63=""),"",VLOOKUP(B63,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B63=""),"",VLOOKUP(B63,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E63" s="25" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F63" s="21" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="G63" s="1" t="n">
         <v>62</v>
@@ -7112,17 +6803,17 @@
         <v>18</v>
       </c>
       <c r="C64" s="9" t="str">
-        <f aca="false">IF((B64=""),"",VLOOKUP(B64,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B64=""),"",VLOOKUP(B64,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D64" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E64" s="25" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="F64" s="21" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="G64" s="1" t="n">
         <v>63</v>
@@ -7136,17 +6827,17 @@
         <v>18</v>
       </c>
       <c r="C65" s="9" t="str">
-        <f aca="false">IF((B65=""),"",VLOOKUP(B65,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B65=""),"",VLOOKUP(B65,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D65" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E65" s="25" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F65" s="21" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G65" s="1" t="n">
         <v>64</v>
@@ -7167,10 +6858,10 @@
         <v>135</v>
       </c>
       <c r="E66" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G66" s="1" t="n">
         <v>65</v>
@@ -7259,7 +6950,9 @@
       <c r="G72" s="1"/>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1"/>
+      <c r="A73" s="1" t="n">
+        <v>72</v>
+      </c>
       <c r="B73" s="12"/>
       <c r="C73" s="9" t="str">
         <f aca="false">IF((B73=""),"",VLOOKUP(B73,Outcomes!$A$2:$D$20,4,0))</f>
@@ -7338,145 +7031,49 @@
       <c r="E80" s="25"/>
       <c r="G80" s="1"/>
     </row>
-    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0"/>
-    </row>
-    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0"/>
-    </row>
-    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="1"/>
-    </row>
-    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="1"/>
-    </row>
-    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="1"/>
-    </row>
-    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="1"/>
-    </row>
-    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1"/>
-    </row>
-    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="1"/>
-      <c r="E88" s="25"/>
-    </row>
-    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="1"/>
-      <c r="E89" s="25"/>
-    </row>
-    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="1"/>
-      <c r="E90" s="25"/>
-    </row>
-    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="1"/>
-      <c r="D91" s="25"/>
-      <c r="E91" s="25"/>
-    </row>
-    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="1"/>
-      <c r="D92" s="25"/>
-      <c r="E92" s="25"/>
-    </row>
-    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="1"/>
-      <c r="D93" s="25"/>
-      <c r="E93" s="25"/>
-    </row>
-    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1"/>
-      <c r="D94" s="25"/>
-      <c r="E94" s="25"/>
-    </row>
-    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="1"/>
-      <c r="D95" s="25"/>
-      <c r="E95" s="25"/>
-    </row>
-    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E96" s="25"/>
-    </row>
-    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D97" s="25"/>
-      <c r="E97" s="25"/>
-    </row>
-    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D98" s="25"/>
-      <c r="E98" s="25"/>
-    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D103" s="25"/>
-      <c r="E103" s="25"/>
-    </row>
-    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E104" s="25"/>
-    </row>
-    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D105" s="25"/>
-      <c r="E105" s="25"/>
-    </row>
-    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D106" s="25"/>
-      <c r="E106" s="25"/>
-    </row>
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E111" s="25"/>
-    </row>
-    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D112" s="25"/>
-    </row>
-    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D113" s="4"/>
-      <c r="E113" s="25"/>
-    </row>
-    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D114" s="25"/>
-      <c r="E114" s="25"/>
-    </row>
-    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E115" s="25"/>
-    </row>
-    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D116" s="25"/>
-      <c r="E116" s="25"/>
-    </row>
-    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D117" s="25"/>
-      <c r="E117" s="25"/>
-    </row>
-    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E118" s="25"/>
-    </row>
-    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D119" s="25"/>
-      <c r="E119" s="25"/>
-    </row>
-    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D120" s="25"/>
-      <c r="E120" s="25"/>
-    </row>
-    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D121" s="25"/>
-      <c r="E121" s="25"/>
-    </row>
-    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E122" s="25"/>
-    </row>
-    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D123" s="25"/>
-      <c r="E123" s="25"/>
-    </row>
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -7492,18 +7089,18 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B35 B37:B41 B45:B56 B58:B62 B66:B80" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B35 B37:B41 B45:B56 B58:B62 B66:B80" type="list">
       <formula1>Outcomes!$A$2:$A$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B36 B42:B44 B57 B63:B65" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B36 B42:B44 B57 B63:B65" type="list">
       <formula1>Outcomes!$A$2:$A$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7517,116 +7114,116 @@
     <tabColor rgb="FFFFF2CC"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BG329"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BG39"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="27" width="24.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="27" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="27" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="27" width="24.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="27" width="16.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="27" width="30.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="27" width="22.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="22" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="59" min="59" style="27" width="8.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="60" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="26" width="24.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="26" width="12.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="26" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="26" width="24.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="26" width="16.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="26" width="30.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="26" width="22.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="22" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="59" min="59" style="26" width="8.87"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="60" style="2" width="8.87"/>
   </cols>
   <sheetData>
-    <row r="1" s="27" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1" s="26" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="28"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="E2" s="28"/>
+        <v>180</v>
+      </c>
+      <c r="E2" s="27"/>
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
       <c r="I2" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="J2" s="28"/>
+        <v>181</v>
+      </c>
+      <c r="J2" s="27"/>
       <c r="K2" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="L2" s="28"/>
+        <v>182</v>
+      </c>
+      <c r="L2" s="27"/>
       <c r="M2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="28"/>
+      <c r="N2" s="27"/>
       <c r="O2" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="P2" s="28"/>
+      <c r="P2" s="27"/>
       <c r="Q2" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="R2" s="28"/>
+        <v>183</v>
+      </c>
+      <c r="R2" s="27"/>
       <c r="S2" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="T2" s="28"/>
+        <v>184</v>
+      </c>
+      <c r="T2" s="27"/>
       <c r="U2" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="V2" s="28"/>
-      <c r="W2" s="28"/>
-      <c r="X2" s="28"/>
-      <c r="Y2" s="28"/>
-      <c r="Z2" s="28"/>
-      <c r="AA2" s="28"/>
-      <c r="AB2" s="28"/>
-      <c r="AC2" s="28"/>
-      <c r="AD2" s="28"/>
-      <c r="AE2" s="28"/>
-      <c r="AF2" s="28"/>
-      <c r="AG2" s="28"/>
-      <c r="AH2" s="28"/>
-      <c r="AI2" s="28"/>
-      <c r="AJ2" s="28"/>
-      <c r="AK2" s="28"/>
-      <c r="AL2" s="28"/>
-      <c r="AM2" s="28"/>
-      <c r="AN2" s="28"/>
-      <c r="AO2" s="28"/>
-      <c r="AP2" s="28"/>
-      <c r="AQ2" s="28"/>
-      <c r="AR2" s="28"/>
-      <c r="AS2" s="28"/>
-      <c r="AT2" s="28"/>
-      <c r="AU2" s="28"/>
-      <c r="AV2" s="28"/>
-      <c r="AW2" s="28"/>
-      <c r="AX2" s="28"/>
-      <c r="AY2" s="28"/>
-      <c r="AZ2" s="28"/>
-      <c r="BA2" s="28"/>
-      <c r="BB2" s="28"/>
-      <c r="BC2" s="28"/>
-      <c r="BD2" s="28"/>
-      <c r="BE2" s="28"/>
-      <c r="BF2" s="28"/>
-      <c r="BG2" s="28"/>
+        <v>185</v>
+      </c>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="27"/>
+      <c r="Y2" s="27"/>
+      <c r="Z2" s="27"/>
+      <c r="AA2" s="27"/>
+      <c r="AB2" s="27"/>
+      <c r="AC2" s="27"/>
+      <c r="AD2" s="27"/>
+      <c r="AE2" s="27"/>
+      <c r="AF2" s="27"/>
+      <c r="AG2" s="27"/>
+      <c r="AH2" s="27"/>
+      <c r="AI2" s="27"/>
+      <c r="AJ2" s="27"/>
+      <c r="AK2" s="27"/>
+      <c r="AL2" s="27"/>
+      <c r="AM2" s="27"/>
+      <c r="AN2" s="27"/>
+      <c r="AO2" s="27"/>
+      <c r="AP2" s="27"/>
+      <c r="AQ2" s="27"/>
+      <c r="AR2" s="27"/>
+      <c r="AS2" s="27"/>
+      <c r="AT2" s="27"/>
+      <c r="AU2" s="27"/>
+      <c r="AV2" s="27"/>
+      <c r="AW2" s="27"/>
+      <c r="AX2" s="27"/>
+      <c r="AY2" s="27"/>
+      <c r="AZ2" s="27"/>
+      <c r="BA2" s="27"/>
+      <c r="BB2" s="27"/>
+      <c r="BC2" s="27"/>
+      <c r="BD2" s="27"/>
+      <c r="BE2" s="27"/>
+      <c r="BF2" s="27"/>
+      <c r="BG2" s="27"/>
     </row>
     <row r="3" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
@@ -7639,11 +7236,11 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>27</v>
@@ -7652,7 +7249,7 @@
         <v>29</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>28</v>
@@ -7667,16 +7264,16 @@
     </row>
     <row r="4" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F4" s="2" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H4" s="29" t="s">
+      <c r="H4" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -7689,7 +7286,7 @@
         <v>36</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>33</v>
@@ -7699,21 +7296,21 @@
         <v>0</v>
       </c>
       <c r="U4" s="25" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="H5" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="H5" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>43</v>
@@ -7722,43 +7319,43 @@
         <v>39</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="U5" s="25" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="H6" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="H6" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>79</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="U6" s="25" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="H7" s="29" t="s">
+        <v>201</v>
+      </c>
+      <c r="H7" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I7" s="2" t="s">
@@ -7768,7 +7365,7 @@
         <v>54</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>146</v>
@@ -7776,9 +7373,9 @@
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H8" s="29" t="s">
+        <v>203</v>
+      </c>
+      <c r="H8" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -7788,7 +7385,7 @@
         <v>67</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>141</v>
@@ -7796,113 +7393,113 @@
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="H9" s="29" t="s">
+        <v>205</v>
+      </c>
+      <c r="H9" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="U9" s="25" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="H10" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="H10" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="U10" s="25" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="H11" s="29" t="s">
+        <v>213</v>
+      </c>
+      <c r="H11" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="O11" s="30"/>
+      <c r="O11" s="29"/>
       <c r="U11" s="25" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="H12" s="29" t="s">
+        <v>215</v>
+      </c>
+      <c r="H12" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O12" s="30"/>
+      <c r="O12" s="29"/>
       <c r="U12" s="25" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="H13" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="H13" s="28" t="s">
         <v>67</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O13" s="30"/>
+      <c r="O13" s="29"/>
       <c r="U13" s="25" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="H14" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="H14" s="28" t="s">
         <v>67</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="O14" s="30"/>
+      <c r="O14" s="29"/>
       <c r="U14" s="25" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="H15" s="29" t="s">
-        <v>202</v>
+        <v>219</v>
+      </c>
+      <c r="H15" s="28" t="s">
+        <v>207</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="M15" s="30"/>
-      <c r="O15" s="30"/>
+        <v>220</v>
+      </c>
+      <c r="M15" s="29"/>
+      <c r="O15" s="29"/>
       <c r="U15" s="25" t="s">
         <v>135</v>
       </c>
@@ -7911,1237 +7508,257 @@
       <c r="B16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H16" s="29" t="s">
-        <v>202</v>
+      <c r="H16" s="28" t="s">
+        <v>207</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="M16" s="30"/>
+        <v>221</v>
+      </c>
+      <c r="M16" s="29"/>
       <c r="U16" s="25" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H17" s="29" t="s">
+      <c r="H17" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M17" s="30"/>
-      <c r="U17" s="30"/>
+        <v>222</v>
+      </c>
+      <c r="M17" s="29"/>
+      <c r="U17" s="29"/>
     </row>
     <row r="18" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M18" s="30"/>
-      <c r="U18" s="30"/>
+      <c r="M18" s="29"/>
+      <c r="U18" s="29"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H19" s="29" t="s">
+      <c r="H19" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="M19" s="30"/>
-      <c r="U19" s="30"/>
+      <c r="M19" s="29"/>
+      <c r="U19" s="29"/>
     </row>
     <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H20" s="29" t="s">
+      <c r="H20" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="M20" s="30"/>
-      <c r="U20" s="30"/>
+        <v>223</v>
+      </c>
+      <c r="M20" s="29"/>
+      <c r="U20" s="29"/>
     </row>
     <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H21" s="29" t="s">
+      <c r="H21" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="M21" s="30"/>
-      <c r="U21" s="30"/>
+      <c r="M21" s="29"/>
+      <c r="U21" s="29"/>
     </row>
     <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H22" s="29" t="s">
+      <c r="H22" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M22" s="30"/>
-      <c r="U22" s="30"/>
+      <c r="M22" s="29"/>
+      <c r="U22" s="29"/>
     </row>
     <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H23" s="29" t="s">
+      <c r="H23" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="M23" s="30"/>
-      <c r="U23" s="30"/>
+        <v>224</v>
+      </c>
+      <c r="M23" s="29"/>
+      <c r="U23" s="29"/>
     </row>
     <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H24" s="29" t="s">
+      <c r="H24" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="M24" s="30"/>
-      <c r="U24" s="30"/>
+        <v>225</v>
+      </c>
+      <c r="M24" s="29"/>
+      <c r="U24" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H25" s="29" t="s">
+      <c r="H25" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M25" s="30"/>
-      <c r="U25" s="30"/>
+      <c r="M25" s="29"/>
+      <c r="U25" s="29"/>
     </row>
     <row r="26" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H26" s="29" t="s">
+      <c r="H26" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M26" s="30"/>
-      <c r="U26" s="30"/>
+      <c r="M26" s="29"/>
+      <c r="U26" s="29"/>
     </row>
     <row r="27" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H27" s="29" t="s">
+      <c r="H27" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="M27" s="30"/>
-      <c r="U27" s="30"/>
+      <c r="M27" s="29"/>
+      <c r="U27" s="29"/>
     </row>
     <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H28" s="29" t="s">
+      <c r="H28" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="M28" s="30"/>
-      <c r="U28" s="30"/>
+      <c r="M28" s="29"/>
+      <c r="U28" s="29"/>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H29" s="29" t="s">
+      <c r="H29" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M29" s="30"/>
-      <c r="U29" s="30"/>
+      <c r="M29" s="29"/>
+      <c r="U29" s="29"/>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H30" s="29" t="s">
+      <c r="H30" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="M30" s="30"/>
-      <c r="U30" s="30"/>
+      <c r="M30" s="29"/>
+      <c r="U30" s="29"/>
     </row>
     <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H31" s="29" t="s">
+      <c r="H31" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="M31" s="30"/>
-      <c r="U31" s="30"/>
+      <c r="M31" s="29"/>
+      <c r="U31" s="29"/>
     </row>
     <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H32" s="29" t="s">
+      <c r="H32" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="M32" s="30"/>
-      <c r="U32" s="30"/>
+        <v>226</v>
+      </c>
+      <c r="M32" s="29"/>
+      <c r="U32" s="29"/>
     </row>
     <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H33" s="29" t="s">
+      <c r="H33" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="M33" s="30"/>
-      <c r="U33" s="30"/>
+        <v>227</v>
+      </c>
+      <c r="M33" s="29"/>
+      <c r="U33" s="29"/>
     </row>
     <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H34" s="29" t="s">
+      <c r="H34" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M34" s="30"/>
-      <c r="U34" s="30"/>
+      <c r="M34" s="29"/>
+      <c r="U34" s="29"/>
     </row>
     <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H35" s="29" t="s">
-        <v>193</v>
+      <c r="H35" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="M35" s="30"/>
-      <c r="U35" s="30"/>
+        <v>228</v>
+      </c>
+      <c r="M35" s="29"/>
+      <c r="U35" s="29"/>
     </row>
     <row r="36" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H36" s="29" t="s">
-        <v>193</v>
+      <c r="H36" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="M36" s="30"/>
-      <c r="U36" s="30"/>
+        <v>229</v>
+      </c>
+      <c r="M36" s="29"/>
+      <c r="U36" s="29"/>
     </row>
     <row r="37" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H37" s="29" t="s">
-        <v>193</v>
+      <c r="H37" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="M37" s="30"/>
-      <c r="U37" s="30"/>
+        <v>230</v>
+      </c>
+      <c r="M37" s="29"/>
+      <c r="U37" s="29"/>
     </row>
     <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H38" s="29" t="s">
-        <v>193</v>
+      <c r="H38" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="M38" s="30"/>
-      <c r="U38" s="30"/>
+        <v>231</v>
+      </c>
+      <c r="M38" s="29"/>
+      <c r="U38" s="29"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H39" s="29" t="s">
-        <v>193</v>
+      <c r="H39" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M39" s="30"/>
-      <c r="U39" s="30"/>
-    </row>
-    <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M40" s="30"/>
-      <c r="U40" s="30"/>
-    </row>
-    <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M41" s="30"/>
-      <c r="U41" s="30"/>
-    </row>
-    <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M42" s="30"/>
-      <c r="U42" s="30"/>
-    </row>
-    <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M43" s="30"/>
-      <c r="U43" s="30"/>
-    </row>
-    <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M44" s="30"/>
-      <c r="U44" s="30"/>
-    </row>
-    <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M45" s="30"/>
-      <c r="U45" s="30"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M46" s="30"/>
-      <c r="U46" s="30"/>
-    </row>
-    <row r="47" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M47" s="30"/>
-      <c r="U47" s="30"/>
-    </row>
-    <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M48" s="30"/>
-      <c r="U48" s="30"/>
-    </row>
-    <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M49" s="30"/>
-      <c r="U49" s="30"/>
-    </row>
-    <row r="50" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M50" s="30"/>
-      <c r="U50" s="30"/>
-    </row>
-    <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M51" s="30"/>
-      <c r="U51" s="30"/>
-    </row>
-    <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M52" s="30"/>
-      <c r="U52" s="30"/>
-    </row>
-    <row r="53" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M53" s="30"/>
-      <c r="U53" s="30"/>
-    </row>
-    <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M54" s="30"/>
-      <c r="U54" s="30"/>
-    </row>
-    <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M55" s="30"/>
-      <c r="U55" s="30"/>
-    </row>
-    <row r="56" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M56" s="30"/>
-      <c r="U56" s="30"/>
-    </row>
-    <row r="57" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M57" s="30"/>
-      <c r="U57" s="30"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M58" s="30"/>
-      <c r="U58" s="30"/>
-    </row>
-    <row r="59" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M59" s="30"/>
-      <c r="U59" s="30"/>
-    </row>
-    <row r="60" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M60" s="30"/>
-      <c r="U60" s="30"/>
-    </row>
-    <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M61" s="30"/>
-      <c r="U61" s="30"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M62" s="30"/>
-      <c r="U62" s="30"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M63" s="30"/>
-      <c r="U63" s="30"/>
-    </row>
-    <row r="64" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M64" s="30"/>
-      <c r="U64" s="30"/>
-    </row>
-    <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M65" s="30"/>
-      <c r="U65" s="30"/>
-    </row>
-    <row r="66" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M66" s="30"/>
-      <c r="U66" s="30"/>
-    </row>
-    <row r="67" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M67" s="30"/>
-      <c r="U67" s="30"/>
-    </row>
-    <row r="68" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M68" s="30"/>
-      <c r="U68" s="30"/>
-    </row>
-    <row r="69" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M69" s="30"/>
-      <c r="U69" s="30"/>
-    </row>
-    <row r="70" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M70" s="30"/>
-      <c r="U70" s="30"/>
-    </row>
-    <row r="71" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M71" s="30"/>
-      <c r="U71" s="30"/>
-    </row>
-    <row r="72" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M72" s="30"/>
-      <c r="U72" s="30"/>
-    </row>
-    <row r="73" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M73" s="30"/>
-      <c r="U73" s="30"/>
-    </row>
-    <row r="74" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M74" s="30"/>
-      <c r="U74" s="30"/>
-    </row>
-    <row r="75" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M75" s="30"/>
-      <c r="U75" s="30"/>
-    </row>
-    <row r="76" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M76" s="30"/>
-      <c r="U76" s="30"/>
-    </row>
-    <row r="77" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M77" s="30"/>
-      <c r="U77" s="30"/>
-    </row>
-    <row r="78" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M78" s="30"/>
-      <c r="U78" s="30"/>
-    </row>
-    <row r="79" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M79" s="30"/>
-      <c r="U79" s="30"/>
-    </row>
-    <row r="80" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M80" s="30"/>
-      <c r="U80" s="30"/>
-    </row>
-    <row r="81" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M81" s="30"/>
-      <c r="U81" s="30"/>
-    </row>
-    <row r="82" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M82" s="30"/>
-      <c r="U82" s="30"/>
-    </row>
-    <row r="83" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M83" s="30"/>
-      <c r="U83" s="30"/>
-    </row>
-    <row r="84" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M84" s="30"/>
-      <c r="U84" s="30"/>
-    </row>
-    <row r="85" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M85" s="30"/>
-      <c r="U85" s="30"/>
-    </row>
-    <row r="86" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M86" s="30"/>
-      <c r="U86" s="30"/>
-    </row>
-    <row r="87" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M87" s="30"/>
-      <c r="U87" s="30"/>
-    </row>
-    <row r="88" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M88" s="30"/>
-      <c r="U88" s="30"/>
-    </row>
-    <row r="89" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M89" s="30"/>
-      <c r="U89" s="30"/>
-    </row>
-    <row r="90" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M90" s="30"/>
-      <c r="U90" s="30"/>
-    </row>
-    <row r="91" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M91" s="30"/>
-      <c r="U91" s="30"/>
-    </row>
-    <row r="92" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M92" s="30"/>
-      <c r="U92" s="30"/>
-    </row>
-    <row r="93" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M93" s="30"/>
-      <c r="U93" s="30"/>
-    </row>
-    <row r="94" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M94" s="30"/>
-      <c r="U94" s="30"/>
-    </row>
-    <row r="95" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M95" s="30"/>
-      <c r="U95" s="30"/>
-    </row>
-    <row r="96" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M96" s="30"/>
-      <c r="U96" s="30"/>
-    </row>
-    <row r="97" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M97" s="30"/>
-      <c r="U97" s="30"/>
-    </row>
-    <row r="98" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M98" s="30"/>
-      <c r="U98" s="30"/>
-    </row>
-    <row r="99" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M99" s="30"/>
-      <c r="U99" s="30"/>
-    </row>
-    <row r="100" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M100" s="30"/>
-      <c r="U100" s="30"/>
-    </row>
-    <row r="101" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M101" s="30"/>
-      <c r="U101" s="30"/>
-    </row>
-    <row r="102" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M102" s="30"/>
-      <c r="U102" s="30"/>
-    </row>
-    <row r="103" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M103" s="30"/>
-      <c r="U103" s="30"/>
-    </row>
-    <row r="104" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M104" s="30"/>
-      <c r="U104" s="30"/>
-    </row>
-    <row r="105" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M105" s="30"/>
-      <c r="U105" s="30"/>
-    </row>
-    <row r="106" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M106" s="30"/>
-      <c r="U106" s="30"/>
-    </row>
-    <row r="107" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M107" s="30"/>
-      <c r="U107" s="30"/>
-    </row>
-    <row r="108" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M108" s="30"/>
-      <c r="U108" s="30"/>
-    </row>
-    <row r="109" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M109" s="30"/>
-      <c r="U109" s="30"/>
-    </row>
-    <row r="110" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M110" s="30"/>
-      <c r="U110" s="30"/>
-    </row>
-    <row r="111" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M111" s="30"/>
-      <c r="U111" s="30"/>
-    </row>
-    <row r="112" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M112" s="30"/>
-      <c r="U112" s="30"/>
-    </row>
-    <row r="113" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M113" s="30"/>
-      <c r="U113" s="30"/>
-    </row>
-    <row r="114" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M114" s="30"/>
-      <c r="U114" s="30"/>
-    </row>
-    <row r="115" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M115" s="30"/>
-      <c r="U115" s="30"/>
-    </row>
-    <row r="116" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M116" s="30"/>
-      <c r="U116" s="30"/>
-    </row>
-    <row r="117" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M117" s="30"/>
-      <c r="U117" s="30"/>
-    </row>
-    <row r="118" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M118" s="30"/>
-      <c r="U118" s="30"/>
-    </row>
-    <row r="119" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M119" s="30"/>
-      <c r="U119" s="30"/>
-    </row>
-    <row r="120" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M120" s="30"/>
-      <c r="U120" s="30"/>
-    </row>
-    <row r="121" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M121" s="30"/>
-      <c r="U121" s="30"/>
-    </row>
-    <row r="122" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M122" s="30"/>
-      <c r="U122" s="30"/>
-    </row>
-    <row r="123" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M123" s="30"/>
-      <c r="U123" s="30"/>
-    </row>
-    <row r="124" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M124" s="30"/>
-      <c r="U124" s="30"/>
-    </row>
-    <row r="125" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M125" s="30"/>
-      <c r="U125" s="30"/>
-    </row>
-    <row r="126" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M126" s="30"/>
-      <c r="U126" s="30"/>
-    </row>
-    <row r="127" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M127" s="30"/>
-      <c r="U127" s="30"/>
-    </row>
-    <row r="128" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M128" s="30"/>
-      <c r="U128" s="30"/>
-    </row>
-    <row r="129" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M129" s="30"/>
-      <c r="U129" s="30"/>
-    </row>
-    <row r="130" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M130" s="30"/>
-      <c r="U130" s="30"/>
-    </row>
-    <row r="131" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M131" s="30"/>
-      <c r="U131" s="30"/>
-    </row>
-    <row r="132" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M132" s="30"/>
-      <c r="U132" s="30"/>
-    </row>
-    <row r="133" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M133" s="30"/>
-      <c r="U133" s="30"/>
-    </row>
-    <row r="134" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M134" s="30"/>
-      <c r="U134" s="30"/>
-    </row>
-    <row r="135" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M135" s="30"/>
-      <c r="U135" s="30"/>
-    </row>
-    <row r="136" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M136" s="30"/>
-      <c r="U136" s="30"/>
-    </row>
-    <row r="137" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M137" s="30"/>
-      <c r="U137" s="30"/>
-    </row>
-    <row r="138" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M138" s="30"/>
-      <c r="U138" s="30"/>
-    </row>
-    <row r="139" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M139" s="30"/>
-      <c r="U139" s="30"/>
-    </row>
-    <row r="140" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M140" s="30"/>
-      <c r="U140" s="30"/>
-    </row>
-    <row r="141" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M141" s="30"/>
-      <c r="U141" s="30"/>
-    </row>
-    <row r="142" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M142" s="30"/>
-      <c r="U142" s="30"/>
-    </row>
-    <row r="143" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M143" s="30"/>
-      <c r="U143" s="30"/>
-    </row>
-    <row r="144" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M144" s="30"/>
-      <c r="U144" s="30"/>
-    </row>
-    <row r="145" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M145" s="30"/>
-      <c r="U145" s="30"/>
-    </row>
-    <row r="146" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M146" s="30"/>
-      <c r="U146" s="30"/>
-    </row>
-    <row r="147" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M147" s="30"/>
-      <c r="U147" s="30"/>
-    </row>
-    <row r="148" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M148" s="30"/>
-      <c r="U148" s="30"/>
-    </row>
-    <row r="149" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M149" s="30"/>
-      <c r="U149" s="30"/>
-    </row>
-    <row r="150" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M150" s="30"/>
-    </row>
-    <row r="151" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M151" s="30"/>
-    </row>
-    <row r="152" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M152" s="30"/>
-    </row>
-    <row r="153" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M153" s="30"/>
-    </row>
-    <row r="154" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M154" s="30"/>
-    </row>
-    <row r="155" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M155" s="30"/>
-    </row>
-    <row r="156" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M156" s="30"/>
-    </row>
-    <row r="157" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M157" s="30"/>
-    </row>
-    <row r="158" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M158" s="30"/>
-    </row>
-    <row r="159" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M159" s="30"/>
-    </row>
-    <row r="160" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M160" s="30"/>
-    </row>
-    <row r="161" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M161" s="30"/>
-    </row>
-    <row r="162" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M162" s="30"/>
-    </row>
-    <row r="163" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M163" s="30"/>
-    </row>
-    <row r="164" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M164" s="30"/>
-    </row>
-    <row r="165" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M165" s="30"/>
-    </row>
-    <row r="166" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M166" s="30"/>
-    </row>
-    <row r="167" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M167" s="30"/>
-    </row>
-    <row r="168" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M168" s="30"/>
-    </row>
-    <row r="169" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M169" s="30"/>
-    </row>
-    <row r="170" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M170" s="30"/>
-    </row>
-    <row r="171" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M171" s="30"/>
-    </row>
-    <row r="172" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M172" s="30"/>
-    </row>
-    <row r="173" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M173" s="30"/>
-    </row>
-    <row r="174" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M174" s="30"/>
-    </row>
-    <row r="175" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M175" s="30"/>
-    </row>
-    <row r="176" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M176" s="30"/>
-    </row>
-    <row r="177" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M177" s="30"/>
-    </row>
-    <row r="178" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M178" s="30"/>
-    </row>
-    <row r="179" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M179" s="30"/>
-    </row>
-    <row r="180" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M180" s="30"/>
-    </row>
-    <row r="181" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M181" s="30"/>
-    </row>
-    <row r="182" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M182" s="30"/>
-    </row>
-    <row r="183" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M183" s="30"/>
-    </row>
-    <row r="184" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M184" s="30"/>
-    </row>
-    <row r="185" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M185" s="30"/>
-    </row>
-    <row r="186" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M186" s="30"/>
-    </row>
-    <row r="187" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M187" s="30"/>
-    </row>
-    <row r="188" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M188" s="30"/>
-    </row>
-    <row r="189" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M189" s="30"/>
-    </row>
-    <row r="190" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M190" s="30"/>
-    </row>
-    <row r="191" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M191" s="30"/>
-    </row>
-    <row r="192" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M192" s="30"/>
-    </row>
-    <row r="193" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M193" s="30"/>
-    </row>
-    <row r="194" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M194" s="30"/>
-    </row>
-    <row r="195" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M195" s="30"/>
-    </row>
-    <row r="196" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M196" s="30"/>
-    </row>
-    <row r="197" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M197" s="30"/>
-    </row>
-    <row r="198" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M198" s="30"/>
-    </row>
-    <row r="199" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M199" s="30"/>
-    </row>
-    <row r="200" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M200" s="30"/>
-    </row>
-    <row r="201" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M201" s="30"/>
-    </row>
-    <row r="202" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M202" s="30"/>
-    </row>
-    <row r="203" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M203" s="30"/>
-    </row>
-    <row r="204" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M204" s="30"/>
-    </row>
-    <row r="205" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M205" s="30"/>
-    </row>
-    <row r="206" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M206" s="30"/>
-    </row>
-    <row r="207" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M207" s="30"/>
-    </row>
-    <row r="208" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M208" s="30"/>
-    </row>
-    <row r="209" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M209" s="30"/>
-    </row>
-    <row r="210" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M210" s="30"/>
-    </row>
-    <row r="211" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M211" s="30"/>
-    </row>
-    <row r="212" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M212" s="30"/>
-    </row>
-    <row r="213" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M213" s="30"/>
-    </row>
-    <row r="214" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M214" s="30"/>
-    </row>
-    <row r="215" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M215" s="30"/>
-    </row>
-    <row r="216" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M216" s="30"/>
-    </row>
-    <row r="217" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M217" s="30"/>
-    </row>
-    <row r="218" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M218" s="30"/>
-    </row>
-    <row r="219" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M219" s="30"/>
-    </row>
-    <row r="220" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M220" s="30"/>
-    </row>
-    <row r="221" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M221" s="30"/>
-    </row>
-    <row r="222" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M222" s="30"/>
-    </row>
-    <row r="223" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M223" s="30"/>
-    </row>
-    <row r="224" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M224" s="30"/>
-    </row>
-    <row r="225" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M225" s="30"/>
-    </row>
-    <row r="226" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M226" s="30"/>
-    </row>
-    <row r="227" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M227" s="30"/>
-    </row>
-    <row r="228" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M228" s="30"/>
-    </row>
-    <row r="229" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M229" s="30"/>
-    </row>
-    <row r="230" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M230" s="30"/>
-    </row>
-    <row r="231" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M231" s="30"/>
-    </row>
-    <row r="232" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M232" s="30"/>
-    </row>
-    <row r="233" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M233" s="30"/>
-    </row>
-    <row r="234" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M234" s="30"/>
-    </row>
-    <row r="235" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M235" s="30"/>
-    </row>
-    <row r="236" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M236" s="30"/>
-    </row>
-    <row r="237" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M237" s="30"/>
-    </row>
-    <row r="238" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M238" s="30"/>
-    </row>
-    <row r="239" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M239" s="30"/>
-    </row>
-    <row r="240" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M240" s="30"/>
-    </row>
-    <row r="241" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M241" s="30"/>
-    </row>
-    <row r="242" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M242" s="30"/>
-    </row>
-    <row r="243" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M243" s="30"/>
-    </row>
-    <row r="244" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M244" s="30"/>
-    </row>
-    <row r="245" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M245" s="30"/>
-    </row>
-    <row r="246" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M246" s="30"/>
-    </row>
-    <row r="247" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M247" s="30"/>
-    </row>
-    <row r="248" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M248" s="30"/>
-    </row>
-    <row r="249" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M249" s="30"/>
-    </row>
-    <row r="250" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M250" s="30"/>
-    </row>
-    <row r="251" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M251" s="30"/>
-    </row>
-    <row r="252" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M252" s="30"/>
-    </row>
-    <row r="253" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M253" s="30"/>
-    </row>
-    <row r="254" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M254" s="30"/>
-    </row>
-    <row r="255" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M255" s="30"/>
-    </row>
-    <row r="256" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M256" s="30"/>
-    </row>
-    <row r="257" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M257" s="30"/>
-    </row>
-    <row r="258" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M258" s="30"/>
-    </row>
-    <row r="259" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M259" s="30"/>
-    </row>
-    <row r="260" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M260" s="30"/>
-    </row>
-    <row r="261" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M261" s="30"/>
-    </row>
-    <row r="262" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M262" s="30"/>
-    </row>
-    <row r="263" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M263" s="30"/>
-    </row>
-    <row r="264" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M264" s="30"/>
-    </row>
-    <row r="265" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M265" s="30"/>
-    </row>
-    <row r="266" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M266" s="30"/>
-    </row>
-    <row r="267" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M267" s="30"/>
-    </row>
-    <row r="268" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M268" s="30"/>
-    </row>
-    <row r="269" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M269" s="30"/>
-    </row>
-    <row r="270" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M270" s="30"/>
-    </row>
-    <row r="271" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M271" s="30"/>
-    </row>
-    <row r="272" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M272" s="30"/>
-    </row>
-    <row r="273" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M273" s="30"/>
-    </row>
-    <row r="274" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M274" s="30"/>
-    </row>
-    <row r="275" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M275" s="30"/>
-    </row>
-    <row r="276" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M276" s="30"/>
-    </row>
-    <row r="277" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M277" s="30"/>
-    </row>
-    <row r="278" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M278" s="30"/>
-    </row>
-    <row r="279" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M279" s="30"/>
-    </row>
-    <row r="280" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M280" s="30"/>
-    </row>
-    <row r="281" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M281" s="30"/>
-    </row>
-    <row r="282" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M282" s="30"/>
-    </row>
-    <row r="283" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M283" s="30"/>
-    </row>
-    <row r="284" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M284" s="30"/>
-    </row>
-    <row r="285" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M285" s="30"/>
-    </row>
-    <row r="286" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M286" s="30"/>
-    </row>
-    <row r="287" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M287" s="30"/>
-    </row>
-    <row r="288" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M288" s="30"/>
-    </row>
-    <row r="289" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M289" s="30"/>
-    </row>
-    <row r="290" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M290" s="30"/>
-    </row>
-    <row r="291" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M291" s="30"/>
-    </row>
-    <row r="292" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M292" s="30"/>
-    </row>
-    <row r="293" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M293" s="30"/>
-    </row>
-    <row r="294" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M294" s="30"/>
-    </row>
-    <row r="295" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M295" s="30"/>
-    </row>
-    <row r="296" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M296" s="30"/>
-    </row>
-    <row r="297" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M297" s="30"/>
-    </row>
-    <row r="298" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M298" s="30"/>
-    </row>
-    <row r="299" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M299" s="30"/>
-    </row>
-    <row r="300" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M300" s="30"/>
-    </row>
-    <row r="301" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M301" s="30"/>
-    </row>
-    <row r="302" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M302" s="30"/>
-    </row>
-    <row r="303" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M303" s="30"/>
-    </row>
-    <row r="304" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M304" s="30"/>
-    </row>
-    <row r="305" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M305" s="30"/>
-    </row>
-    <row r="306" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M306" s="30"/>
-    </row>
-    <row r="307" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M307" s="30"/>
-    </row>
-    <row r="308" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M308" s="30"/>
-    </row>
-    <row r="309" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M309" s="30"/>
-    </row>
-    <row r="310" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M310" s="30"/>
-    </row>
-    <row r="311" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M311" s="30"/>
-    </row>
-    <row r="312" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M312" s="30"/>
-    </row>
-    <row r="313" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M313" s="30"/>
-    </row>
-    <row r="314" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M314" s="30"/>
-    </row>
-    <row r="315" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M315" s="30"/>
-    </row>
-    <row r="316" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M316" s="30"/>
-    </row>
-    <row r="317" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M317" s="30"/>
-    </row>
-    <row r="318" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M318" s="30"/>
-    </row>
-    <row r="319" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M319" s="30"/>
-    </row>
-    <row r="320" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M320" s="30"/>
-    </row>
-    <row r="321" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M321" s="30"/>
-    </row>
-    <row r="322" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M322" s="30"/>
-    </row>
-    <row r="323" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M323" s="30"/>
-    </row>
-    <row r="324" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M324" s="30"/>
-    </row>
-    <row r="325" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M325" s="30"/>
-    </row>
-    <row r="326" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M326" s="30"/>
-    </row>
-    <row r="327" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M327" s="30"/>
-    </row>
-    <row r="328" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M328" s="30"/>
-    </row>
-    <row r="329" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M329" s="30"/>
+      <c r="M39" s="29"/>
+      <c r="U39" s="29"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H3:H39" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H3:H39" type="list">
       <formula1>$K$3:$K$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9158,15 +7775,15 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="2.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="2"/>
   </cols>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9183,8 +7800,8 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>

<commit_message>
[Track-619] update project notification template and actions (#2744)
</commit_message>
<xml_diff>
--- a/epictrack-api/src/api/templates/event_templates/project_notification/003_Project_Notification.xlsx
+++ b/epictrack-api/src/api/templates/event_templates/project_notification/003_Project_Notification.xlsx
@@ -16,9 +16,6 @@
     <sheet name="Outcome_Temp" sheetId="6" state="visible" r:id="rId7"/>
     <sheet name="Action_Temp" sheetId="7" state="visible" r:id="rId8"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId9"/>
-  </externalReferences>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Events!$A$1:$M$62</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Outcomes!$A$1:$F$15</definedName>
@@ -33,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="232">
   <si>
     <t xml:space="preserve">No</t>
   </si>
@@ -444,7 +441,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Decision: Project Notification", "new_name": "Decision: Project Notification" }</t>
+    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Decision: Project Notification", "new_name": "Decision: Project Notification","use_phase_start":"True" }</t>
   </si>
   <si>
     <r>
@@ -499,7 +496,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Notification Decision Announcement &amp; Tweet", "new_name": "Notification Decision Announcement &amp; Tweet" }</t>
+    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Notification Decision Announcement &amp; Tweet", "new_name": "Notification Decision Announcement &amp; Tweet", "use_phase_start":"True" }</t>
   </si>
   <si>
     <r>
@@ -554,42 +551,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Executive Calendar Notification", "new_name": "Executive Calendar Notification" }</t>
+    <t xml:space="preserve">{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Executive Calendar Notification", "new_name": "Executive Calendar Notification","use_phase_start":"True" }</t>
   </si>
   <si>
     <t xml:space="preserve">SetEventsStatus</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Set “Notification Review | </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Project Notification Report referred to Decision Maker</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">” to INACTIVE</t>
-    </r>
+    <t xml:space="preserve">Set "Notification Review | Project Notification Report referred to Decision Maker" to INACTIVE</t>
   </si>
   <si>
     <t xml:space="preserve">[{"phase_name":"Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Report referred to Decision Maker", "is_active": false }]</t>
@@ -598,7 +566,7 @@
     <t xml:space="preserve">SetPhasesStatus</t>
   </si>
   <si>
-    <t xml:space="preserve">Set finalPhase “Notification Decision” to INACTIVE</t>
+    <t xml:space="preserve">Set finalPhase "Notification Decision" to INACTIVE</t>
   </si>
   <si>
     <t xml:space="preserve">[{"phase_name":"Notification Decision","work_type_id": 1, "ea_act_id": 3, "is_active": false }]</t>
@@ -658,6 +626,18 @@
     <t xml:space="preserve">{"start_date_locked": true}</t>
   </si>
   <si>
+    <t xml:space="preserve">{"work_type_id": 1, "ea_act_id": 3, "event_name": "Decision: Project Notification", "new_name": "Decision: Project Notification", "use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"work_type_id": 1, "ea_act_id": 3, "event_name": "Notification Decision Announcement &amp; Tweet", "new_name": "Notification Decision Announcement &amp; Tweet","use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"work_type_id": 1, "ea_act_id": 3, "event_name": "Executive Calendar Notification", "new_name": "Executive Calendar Notification","use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Report referred to Decision Maker", "is_active": false }]</t>
+  </si>
+  <si>
     <t xml:space="preserve">Set workState to TERMINATED</t>
   </si>
   <si>
@@ -688,59 +668,13 @@
     <t xml:space="preserve">SetEventName</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Rename </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">"Start of Intake Phase (e.g. Initial Contact, Draft Sharing, or PN Submission)" to </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"Start of Revised PN Development"</t>
-    </r>
+    <t xml:space="preserve">Rename "Start of Intake Phase (e.g. Initial Contact, Draft Sharing, or PN Submission)" to "Start of Revised PN Development"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Project Notification Development","work_type_id": 1, "ea_act_id": 3, "event_name": "Start of Intake Phase (e.g. Initial Contact, Draft Sharing, or PN Submission)", "new_name": "Start of Revised PN Development" }</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Rename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> "Last Day of Intake Phase (day before formal submission)" to "Last Day of Revised PN Development Phase (day before re-submission)"</t>
-    </r>
+    <t xml:space="preserve">Rename "Last Day of Intake Phase (day before formal submission)" to "Last Day of Revised PN Development Phase (day before re-submission)"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Project Notification Development","work_type_id": 1, "ea_act_id": 3, "event_name": "Last Day of Intake Phase (day before formal submission)", "new_name": "Last Day of Revised PN Development Phase (day before re-submission)" }</t>
@@ -752,49 +686,13 @@
     <t xml:space="preserve">[{"phase_name":"Revised Project Notification Development","work_type_id": 1, "ea_act_id": 3, "event_name": "Meeting with Proponent", "is_active": false }]</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Rename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> "Project Notification Submission Received (Day Zero)" to "Revised PN Submission Received"</t>
-    </r>
+    <t xml:space="preserve">Rename "Project Notification Submission Received (Day Zero)" to "Revised PN Submission Received"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Submission Received (Day Zero)", "new_name": "Revised PN Submission Received" }</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Rename</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> "Project Notification Report referred to Decision Maker" to "Revised PN Report referred to Decision Maker"</t>
-    </r>
+    <t xml:space="preserve">Rename "Project Notification Report referred to Decision Maker" to "Revised PN Report referred to Decision Maker"</t>
   </si>
   <si>
     <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Project Notification Report referred to Decision Maker", "new_name": "Revised PN Report referred to Decision Maker" } </t>
@@ -809,13 +707,16 @@
     <t xml:space="preserve">AddEvent "Revised Notification Review | Comment Period" and set visibility to SUGGESTED (copy of Comment Period)</t>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Comment Period","visibility": "SUGGESTED" }</t>
+    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Comment Period","visibility": "SUGGESTED", "start_at": "14", "use_phase_start":"True" }</t>
   </si>
   <si>
     <t xml:space="preserve">AddEvent "Revised Notification Review | Delegation of PN Decision" and set visibility to SUGGESTED (renamed copy of Delegation of Decision)</t>
   </si>
   <si>
-    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Delegation of PN Decision", "new_name": "Delegation of PN Decision","visibility": "SUGGESTED", "start_at": 1 }</t>
+    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Delegation of PN Decision", "new_name": "Delegation of PN Decision","visibility": "SUGGESTED", "start_at": "7", "use_phase_start":"True" }</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{"phase_name":"Revised Notification Review","work_type_id": 1, "ea_act_id": 3, "event_name": "Comment Period","visibility": "SUGGESTED", "start_at": "14", "use_phase_start":"True"}</t>
   </si>
   <si>
     <t xml:space="preserve">EA Act</t>
@@ -982,7 +883,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1040,12 +941,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -1156,7 +1051,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1261,10 +1156,6 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1290,7 +1181,92 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="15">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCCCCC"/>
+          <bgColor rgb="FF272727"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2E75B6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCCCCFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF3F3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFBE5D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="1"/>
@@ -1312,6 +1288,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF2F75B5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1387,305 +1370,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Phases"/>
-      <sheetName val="Events"/>
-      <sheetName val="Outcomes"/>
-      <sheetName val="Actions"/>
-      <sheetName val="Lookups"/>
-      <sheetName val="Outcome_Temp"/>
-      <sheetName val="Action_Temp"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2">
-        <row r="2">
-          <cell r="A2">
-            <v>1</v>
-          </cell>
-          <cell r="B2">
-            <v>6</v>
-          </cell>
-          <cell r="C2" t="str">
-            <v>EAO's Viewpoint on Submitted Document</v>
-          </cell>
-          <cell r="D2" t="str">
-            <v>Viewpoint is POSITIVE</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="A3">
-            <v>2</v>
-          </cell>
-          <cell r="B3">
-            <v>6</v>
-          </cell>
-          <cell r="C3" t="str">
-            <v>EAO's Viewpoint on Submitted Document</v>
-          </cell>
-          <cell r="D3" t="str">
-            <v>Viewpoint is NEGATIVE</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="A4">
-            <v>3</v>
-          </cell>
-          <cell r="B4">
-            <v>7</v>
-          </cell>
-          <cell r="C4" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D4" t="str">
-            <v>Minister's Decision</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5">
-            <v>4</v>
-          </cell>
-          <cell r="B5">
-            <v>7</v>
-          </cell>
-          <cell r="C5" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D5" t="str">
-            <v>CEAO's Decision</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6">
-            <v>5</v>
-          </cell>
-          <cell r="B6">
-            <v>8</v>
-          </cell>
-          <cell r="C6" t="str">
-            <v>Project Notification Withdrawn</v>
-          </cell>
-          <cell r="D6" t="str">
-            <v>PN Submission Withdrawn</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7">
-            <v>6</v>
-          </cell>
-          <cell r="B7">
-            <v>9</v>
-          </cell>
-          <cell r="C7" t="str">
-            <v>Direct Submission of Project Notification - DELETE this Intake Phase!</v>
-          </cell>
-          <cell r="D7" t="str">
-            <v>Delete the Intake Phase</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8">
-            <v>7</v>
-          </cell>
-          <cell r="B8">
-            <v>12</v>
-          </cell>
-          <cell r="C8" t="str">
-            <v>Project Notification Submission Received (Day Zero)</v>
-          </cell>
-          <cell r="D8" t="str">
-            <v>Start the Review Period</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9">
-            <v>8</v>
-          </cell>
-          <cell r="B9">
-            <v>14</v>
-          </cell>
-          <cell r="C9" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D9" t="str">
-            <v>Minister's Decision</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10">
-            <v>9</v>
-          </cell>
-          <cell r="B10">
-            <v>14</v>
-          </cell>
-          <cell r="C10" t="str">
-            <v>Delegation of PN Decision</v>
-          </cell>
-          <cell r="D10" t="str">
-            <v>CEAO's Decision</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11">
-            <v>10</v>
-          </cell>
-          <cell r="B11">
-            <v>36</v>
-          </cell>
-          <cell r="C11" t="str">
-            <v>Project Notification Terminated s.39(d)</v>
-          </cell>
-          <cell r="D11" t="str">
-            <v>PN is Terminated (s.39)</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12">
-            <v>11</v>
-          </cell>
-          <cell r="B12">
-            <v>39</v>
-          </cell>
-          <cell r="C12" t="str">
-            <v>Project Notification Withdrawn</v>
-          </cell>
-          <cell r="D12" t="str">
-            <v>PN Submission Withdrawn</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13">
-            <v>12</v>
-          </cell>
-          <cell r="B13">
-            <v>44</v>
-          </cell>
-          <cell r="C13" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D13" t="str">
-            <v>No Further Review Required</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14">
-            <v>13</v>
-          </cell>
-          <cell r="B14">
-            <v>44</v>
-          </cell>
-          <cell r="C14" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D14" t="str">
-            <v>Revised PN Submission Required</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15">
-            <v>14</v>
-          </cell>
-          <cell r="B15">
-            <v>44</v>
-          </cell>
-          <cell r="C15" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D15" t="str">
-            <v>Referred for Minister's Designation</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16">
-            <v>15</v>
-          </cell>
-          <cell r="B16">
-            <v>52</v>
-          </cell>
-          <cell r="C16" t="str">
-            <v>Project Notification Terminated s.39(d)</v>
-          </cell>
-          <cell r="D16" t="str">
-            <v>PN is Terminated (s.39)</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17">
-            <v>16</v>
-          </cell>
-          <cell r="B17">
-            <v>55</v>
-          </cell>
-          <cell r="C17" t="str">
-            <v>Project Notification Withdrawn</v>
-          </cell>
-          <cell r="D17" t="str">
-            <v>PN Submission Withdrawn</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18">
-            <v>17</v>
-          </cell>
-          <cell r="B18">
-            <v>59</v>
-          </cell>
-          <cell r="C18" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D18" t="str">
-            <v>No Further Review Required</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19">
-            <v>18</v>
-          </cell>
-          <cell r="B19">
-            <v>59</v>
-          </cell>
-          <cell r="C19" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D19" t="str">
-            <v>Revised PN Submission Required</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20">
-            <v>19</v>
-          </cell>
-          <cell r="B20">
-            <v>59</v>
-          </cell>
-          <cell r="C20" t="str">
-            <v>Decision: Project Notification</v>
-          </cell>
-          <cell r="D20" t="str">
-            <v>Referred for Minister's Designation</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="50.67"/>
@@ -1693,7 +1384,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="14.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="2" width="12.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="10.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1769,7 +1460,7 @@
         <v>11</v>
       </c>
       <c r="E3" s="1" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F3" s="6" t="n">
         <f aca="false">TRUE()</f>
@@ -1817,22 +1508,22 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C4" type="list">
       <formula1>Lookups!$B$3:$B$16</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D2:D4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="D2:D4" type="list">
       <formula1>Lookups!$D$3:$D$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F4" type="list">
       <formula1>Lookups!$F$3:$F$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1846,21 +1537,21 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M62"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="51.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="17.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="51.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="17.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="13.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="14.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="9.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="3.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="11.36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="3.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="11.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="2" width="14.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="2" width="10.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="14" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="14" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2178,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K8" s="1" t="n">
         <v>0</v>
@@ -2587,7 +2278,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1" t="n">
         <v>0</v>
@@ -2922,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="K26" s="1" t="n">
         <v>0</v>
@@ -3644,7 +3335,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
@@ -3672,7 +3363,7 @@
         <v>0</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K44" s="1" t="n">
         <v>0</v>
@@ -3684,7 +3375,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="n">
         <v>44</v>
       </c>
@@ -3712,7 +3403,7 @@
         <v>0</v>
       </c>
       <c r="J45" s="21" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="K45" s="1" t="n">
         <v>0</v>
@@ -4437,46 +4128,46 @@
   </sheetData>
   <autoFilter ref="A1:M62"/>
   <conditionalFormatting sqref="H1:H62">
-    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="END" dxfId="0">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="END" dxfId="12">
       <formula>NOT(ISERROR(SEARCH("END",H1)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="START" dxfId="1">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="START" dxfId="13">
       <formula>NOT(ISERROR(SEARCH("START",H1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F2:F62" type="list">
       <formula1>Lookups!$I$3:$I$39</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="I2:I62" type="list">
       <formula1>Lookups!$S$3:$S$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G2:G62" type="list">
       <formula1>Lookups!$K$3:$K$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C2:C62" type="list">
       <formula1>Phases!$A$2:$A$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L2:L3 L5:L62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L2:L3 L5:L62" type="list">
       <formula1>Lookups!$M$3:$M$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H2:H62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H2:H62" type="list">
       <formula1>Lookups!$Q$3:$Q$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L4" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="L4" type="list">
       <formula1>Lookups!$M$3:$M$6</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4491,15 +4182,15 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F72"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="6.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="30.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="70.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="70.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="7" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="7" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5559,14 +5250,14 @@
   </sheetData>
   <autoFilter ref="A1:F15"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B57" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B57" type="list">
       <formula1>Events!$A$2:$A$62</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5581,16 +5272,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G1048576"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="7.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="70.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="18.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="116.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="63.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="87.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="12.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="8" style="2" width="8.87"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5736,7 +5427,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
@@ -5760,7 +5451,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
@@ -6042,7 +5733,7 @@
         <v>119</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>18</v>
@@ -6066,7 +5757,7 @@
         <v>121</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>122</v>
+        <v>150</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>19</v>
@@ -6090,13 +5781,13 @@
         <v>123</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>124</v>
+        <v>151</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
@@ -6114,13 +5805,13 @@
         <v>126</v>
       </c>
       <c r="F22" s="21" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
@@ -6231,10 +5922,10 @@
         <v>135</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G27" s="1" t="n">
         <v>26</v>
@@ -6375,10 +6066,10 @@
         <v>135</v>
       </c>
       <c r="E33" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G33" s="1" t="n">
         <v>32</v>
@@ -6408,7 +6099,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
         <v>34</v>
       </c>
@@ -6420,13 +6111,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E35" s="25" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F35" s="21" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G35" s="1" t="n">
         <v>34</v>
@@ -6440,23 +6131,23 @@
         <v>13</v>
       </c>
       <c r="C36" s="9" t="str">
-        <f aca="false">IF((B36=""),"",VLOOKUP(B36,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B36=""),"",VLOOKUP(B36,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D36" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E36" s="25" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F36" s="21" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="G36" s="1" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
@@ -6468,19 +6159,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G37" s="1" t="n">
         <v>36</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="n">
         <v>37</v>
       </c>
@@ -6492,13 +6183,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E38" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
+      </c>
+      <c r="E38" s="25" t="s">
+        <v>165</v>
       </c>
       <c r="F38" s="21" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G38" s="1" t="n">
         <v>37</v>
@@ -6519,16 +6210,16 @@
         <v>125</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F39" s="21" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G39" s="1" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
@@ -6540,19 +6231,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E40" s="26" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="F40" s="21" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="G40" s="1" t="n">
         <v>39</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="n">
         <v>40</v>
       </c>
@@ -6564,13 +6255,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E41" s="26" t="s">
-        <v>167</v>
+        <v>162</v>
+      </c>
+      <c r="E41" s="25" t="s">
+        <v>171</v>
       </c>
       <c r="F41" s="21" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G41" s="1" t="n">
         <v>40</v>
@@ -6584,17 +6275,17 @@
         <v>13</v>
       </c>
       <c r="C42" s="9" t="str">
-        <f aca="false">IF((B42=""),"",VLOOKUP(B42,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B42=""),"",VLOOKUP(B42,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E42" s="25" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F42" s="21" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="G42" s="1" t="n">
         <v>41</v>
@@ -6608,17 +6299,17 @@
         <v>13</v>
       </c>
       <c r="C43" s="9" t="str">
-        <f aca="false">IF((B43=""),"",VLOOKUP(B43,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B43=""),"",VLOOKUP(B43,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D43" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="F43" s="21" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="G43" s="1" t="n">
         <v>42</v>
@@ -6632,17 +6323,17 @@
         <v>13</v>
       </c>
       <c r="C44" s="9" t="str">
-        <f aca="false">IF((B44=""),"",VLOOKUP(B44,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B44=""),"",VLOOKUP(B44,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D44" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E44" s="25" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F44" s="21" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G44" s="1" t="n">
         <v>43</v>
@@ -6663,10 +6354,10 @@
         <v>135</v>
       </c>
       <c r="E45" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G45" s="1" t="n">
         <v>44</v>
@@ -6735,10 +6426,10 @@
         <v>135</v>
       </c>
       <c r="E48" s="25" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F48" s="21" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G48" s="1" t="n">
         <v>47</v>
@@ -6879,10 +6570,10 @@
         <v>135</v>
       </c>
       <c r="E54" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G54" s="1" t="n">
         <v>53</v>
@@ -6912,7 +6603,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="n">
         <v>55</v>
       </c>
@@ -6924,13 +6615,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="E56" s="25" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="F56" s="21" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="G56" s="1" t="n">
         <v>55</v>
@@ -6941,26 +6632,26 @@
         <v>56</v>
       </c>
       <c r="B57" s="12" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C57" s="9" t="str">
-        <f aca="false">IF((B57=""),"",VLOOKUP(B57,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B57=""),"",VLOOKUP(B57,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D57" s="25" t="s">
         <v>141</v>
       </c>
       <c r="E57" s="25" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F57" s="21" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="G57" s="1" t="n">
         <v>56</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="n">
         <v>57</v>
       </c>
@@ -6972,19 +6663,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E58" s="25" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G58" s="1" t="n">
         <v>57</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="n">
         <v>58</v>
       </c>
@@ -6996,13 +6687,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E59" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
+      </c>
+      <c r="E59" s="25" t="s">
+        <v>165</v>
       </c>
       <c r="F59" s="21" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G59" s="1" t="n">
         <v>58</v>
@@ -7023,16 +6714,16 @@
         <v>125</v>
       </c>
       <c r="E60" s="25" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F60" s="21" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="G60" s="1" t="n">
         <v>59</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="n">
         <v>60</v>
       </c>
@@ -7044,19 +6735,19 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E61" s="26" t="s">
-        <v>165</v>
+        <v>162</v>
+      </c>
+      <c r="E61" s="25" t="s">
+        <v>169</v>
       </c>
       <c r="F61" s="21" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="G61" s="1" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="n">
         <v>61</v>
       </c>
@@ -7068,13 +6759,13 @@
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E62" s="26" t="s">
-        <v>167</v>
+        <v>162</v>
+      </c>
+      <c r="E62" s="25" t="s">
+        <v>171</v>
       </c>
       <c r="F62" s="21" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="G62" s="1" t="n">
         <v>61</v>
@@ -7088,17 +6779,17 @@
         <v>18</v>
       </c>
       <c r="C63" s="9" t="str">
-        <f aca="false">IF((B63=""),"",VLOOKUP(B63,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B63=""),"",VLOOKUP(B63,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E63" s="25" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="F63" s="21" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="G63" s="1" t="n">
         <v>62</v>
@@ -7112,17 +6803,17 @@
         <v>18</v>
       </c>
       <c r="C64" s="9" t="str">
-        <f aca="false">IF((B64=""),"",VLOOKUP(B64,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B64=""),"",VLOOKUP(B64,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D64" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E64" s="25" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="F64" s="21" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="G64" s="1" t="n">
         <v>63</v>
@@ -7136,17 +6827,17 @@
         <v>18</v>
       </c>
       <c r="C65" s="9" t="str">
-        <f aca="false">IF((B65=""),"",VLOOKUP(B65,[2]Outcomes!$A$2:$D$20,4,0))</f>
+        <f aca="false">IF((B65=""),"",VLOOKUP(B65,Outcomes!$A$2:$D$20,4,0))</f>
         <v>Revised PN Submission Required</v>
       </c>
       <c r="D65" s="25" t="s">
         <v>118</v>
       </c>
       <c r="E65" s="25" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F65" s="21" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="G65" s="1" t="n">
         <v>64</v>
@@ -7167,10 +6858,10 @@
         <v>135</v>
       </c>
       <c r="E66" s="25" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G66" s="1" t="n">
         <v>65</v>
@@ -7259,7 +6950,9 @@
       <c r="G72" s="1"/>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="1"/>
+      <c r="A73" s="1" t="n">
+        <v>72</v>
+      </c>
       <c r="B73" s="12"/>
       <c r="C73" s="9" t="str">
         <f aca="false">IF((B73=""),"",VLOOKUP(B73,Outcomes!$A$2:$D$20,4,0))</f>
@@ -7338,145 +7031,49 @@
       <c r="E80" s="25"/>
       <c r="G80" s="1"/>
     </row>
-    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="0"/>
-    </row>
-    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="0"/>
-    </row>
-    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="1"/>
-    </row>
-    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="1"/>
-    </row>
-    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="1"/>
-    </row>
-    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="1"/>
-    </row>
-    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="1"/>
-    </row>
-    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="1"/>
-      <c r="E88" s="25"/>
-    </row>
-    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="1"/>
-      <c r="E89" s="25"/>
-    </row>
-    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="1"/>
-      <c r="E90" s="25"/>
-    </row>
-    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="1"/>
-      <c r="D91" s="25"/>
-      <c r="E91" s="25"/>
-    </row>
-    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="1"/>
-      <c r="D92" s="25"/>
-      <c r="E92" s="25"/>
-    </row>
-    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="1"/>
-      <c r="D93" s="25"/>
-      <c r="E93" s="25"/>
-    </row>
-    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1"/>
-      <c r="D94" s="25"/>
-      <c r="E94" s="25"/>
-    </row>
-    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="1"/>
-      <c r="D95" s="25"/>
-      <c r="E95" s="25"/>
-    </row>
-    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E96" s="25"/>
-    </row>
-    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D97" s="25"/>
-      <c r="E97" s="25"/>
-    </row>
-    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D98" s="25"/>
-      <c r="E98" s="25"/>
-    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D103" s="25"/>
-      <c r="E103" s="25"/>
-    </row>
-    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E104" s="25"/>
-    </row>
-    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D105" s="25"/>
-      <c r="E105" s="25"/>
-    </row>
-    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D106" s="25"/>
-      <c r="E106" s="25"/>
-    </row>
+    <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E111" s="25"/>
-    </row>
-    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D112" s="25"/>
-    </row>
-    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D113" s="4"/>
-      <c r="E113" s="25"/>
-    </row>
-    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D114" s="25"/>
-      <c r="E114" s="25"/>
-    </row>
-    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E115" s="25"/>
-    </row>
-    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D116" s="25"/>
-      <c r="E116" s="25"/>
-    </row>
-    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D117" s="25"/>
-      <c r="E117" s="25"/>
-    </row>
-    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E118" s="25"/>
-    </row>
-    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D119" s="25"/>
-      <c r="E119" s="25"/>
-    </row>
-    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D120" s="25"/>
-      <c r="E120" s="25"/>
-    </row>
-    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D121" s="25"/>
-      <c r="E121" s="25"/>
-    </row>
-    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E122" s="25"/>
-    </row>
-    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D123" s="25"/>
-      <c r="E123" s="25"/>
-    </row>
+    <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048564" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048565" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048566" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -7492,18 +7089,18 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B35 B37:B41 B45:B56 B58:B62 B66:B80" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B2:B35 B37:B41 B45:B56 B58:B62 B66:B80" type="list">
       <formula1>Outcomes!$A$2:$A$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B36 B42:B44 B57 B63:B65" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="B36 B42:B44 B57 B63:B65" type="list">
       <formula1>Outcomes!$A$2:$A$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7517,116 +7114,116 @@
     <tabColor rgb="FFFFF2CC"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BG329"/>
-  <sheetFormatPr defaultColWidth="8.87890625" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:BG39"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="27" width="24.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="27" width="12.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="27" width="10.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="27" width="24.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="27" width="16.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="27" width="30.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="27" width="14.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="27" width="22.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="22" style="27" width="3.66"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="59" min="59" style="27" width="8.88"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="60" style="2" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="26" width="24.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="26" width="12.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="26" width="10.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="26" width="24.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="26" width="16.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="26" width="30.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="26" width="14.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="26" width="22.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="22" style="26" width="3.65"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="59" min="59" style="26" width="8.87"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="60" style="2" width="8.87"/>
   </cols>
   <sheetData>
-    <row r="1" s="27" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1" s="26" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="2" s="3" customFormat="true" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="28"/>
+      <c r="A2" s="27"/>
       <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="E2" s="28"/>
+        <v>180</v>
+      </c>
+      <c r="E2" s="27"/>
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
       <c r="I2" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="J2" s="28"/>
+        <v>181</v>
+      </c>
+      <c r="J2" s="27"/>
       <c r="K2" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="L2" s="28"/>
+        <v>182</v>
+      </c>
+      <c r="L2" s="27"/>
       <c r="M2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="N2" s="28"/>
+      <c r="N2" s="27"/>
       <c r="O2" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="P2" s="28"/>
+      <c r="P2" s="27"/>
       <c r="Q2" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="R2" s="28"/>
+        <v>183</v>
+      </c>
+      <c r="R2" s="27"/>
       <c r="S2" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="T2" s="28"/>
+        <v>184</v>
+      </c>
+      <c r="T2" s="27"/>
       <c r="U2" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="V2" s="28"/>
-      <c r="W2" s="28"/>
-      <c r="X2" s="28"/>
-      <c r="Y2" s="28"/>
-      <c r="Z2" s="28"/>
-      <c r="AA2" s="28"/>
-      <c r="AB2" s="28"/>
-      <c r="AC2" s="28"/>
-      <c r="AD2" s="28"/>
-      <c r="AE2" s="28"/>
-      <c r="AF2" s="28"/>
-      <c r="AG2" s="28"/>
-      <c r="AH2" s="28"/>
-      <c r="AI2" s="28"/>
-      <c r="AJ2" s="28"/>
-      <c r="AK2" s="28"/>
-      <c r="AL2" s="28"/>
-      <c r="AM2" s="28"/>
-      <c r="AN2" s="28"/>
-      <c r="AO2" s="28"/>
-      <c r="AP2" s="28"/>
-      <c r="AQ2" s="28"/>
-      <c r="AR2" s="28"/>
-      <c r="AS2" s="28"/>
-      <c r="AT2" s="28"/>
-      <c r="AU2" s="28"/>
-      <c r="AV2" s="28"/>
-      <c r="AW2" s="28"/>
-      <c r="AX2" s="28"/>
-      <c r="AY2" s="28"/>
-      <c r="AZ2" s="28"/>
-      <c r="BA2" s="28"/>
-      <c r="BB2" s="28"/>
-      <c r="BC2" s="28"/>
-      <c r="BD2" s="28"/>
-      <c r="BE2" s="28"/>
-      <c r="BF2" s="28"/>
-      <c r="BG2" s="28"/>
+        <v>185</v>
+      </c>
+      <c r="V2" s="27"/>
+      <c r="W2" s="27"/>
+      <c r="X2" s="27"/>
+      <c r="Y2" s="27"/>
+      <c r="Z2" s="27"/>
+      <c r="AA2" s="27"/>
+      <c r="AB2" s="27"/>
+      <c r="AC2" s="27"/>
+      <c r="AD2" s="27"/>
+      <c r="AE2" s="27"/>
+      <c r="AF2" s="27"/>
+      <c r="AG2" s="27"/>
+      <c r="AH2" s="27"/>
+      <c r="AI2" s="27"/>
+      <c r="AJ2" s="27"/>
+      <c r="AK2" s="27"/>
+      <c r="AL2" s="27"/>
+      <c r="AM2" s="27"/>
+      <c r="AN2" s="27"/>
+      <c r="AO2" s="27"/>
+      <c r="AP2" s="27"/>
+      <c r="AQ2" s="27"/>
+      <c r="AR2" s="27"/>
+      <c r="AS2" s="27"/>
+      <c r="AT2" s="27"/>
+      <c r="AU2" s="27"/>
+      <c r="AV2" s="27"/>
+      <c r="AW2" s="27"/>
+      <c r="AX2" s="27"/>
+      <c r="AY2" s="27"/>
+      <c r="AZ2" s="27"/>
+      <c r="BA2" s="27"/>
+      <c r="BB2" s="27"/>
+      <c r="BC2" s="27"/>
+      <c r="BD2" s="27"/>
+      <c r="BE2" s="27"/>
+      <c r="BF2" s="27"/>
+      <c r="BG2" s="27"/>
     </row>
     <row r="3" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
@@ -7639,11 +7236,11 @@
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>27</v>
@@ -7652,7 +7249,7 @@
         <v>29</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>28</v>
@@ -7667,16 +7264,16 @@
     </row>
     <row r="4" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="2" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F4" s="2" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="H4" s="29" t="s">
+      <c r="H4" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I4" s="2" t="s">
@@ -7689,7 +7286,7 @@
         <v>36</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>33</v>
@@ -7699,21 +7296,21 @@
         <v>0</v>
       </c>
       <c r="U4" s="25" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="2" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="H5" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="H5" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>43</v>
@@ -7722,43 +7319,43 @@
         <v>39</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>51</v>
       </c>
       <c r="U5" s="25" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="H6" s="29" t="s">
+        <v>196</v>
+      </c>
+      <c r="H6" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>79</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="U6" s="25" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="H7" s="29" t="s">
+        <v>201</v>
+      </c>
+      <c r="H7" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I7" s="2" t="s">
@@ -7768,7 +7365,7 @@
         <v>54</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="U7" s="25" t="s">
         <v>146</v>
@@ -7776,9 +7373,9 @@
     </row>
     <row r="8" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="H8" s="29" t="s">
+        <v>203</v>
+      </c>
+      <c r="H8" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I8" s="2" t="s">
@@ -7788,7 +7385,7 @@
         <v>67</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="U8" s="25" t="s">
         <v>141</v>
@@ -7796,113 +7393,113 @@
     </row>
     <row r="9" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="H9" s="29" t="s">
+        <v>205</v>
+      </c>
+      <c r="H9" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="U9" s="25" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="H10" s="29" t="s">
+        <v>210</v>
+      </c>
+      <c r="H10" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>38</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="U10" s="25" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="H11" s="29" t="s">
+        <v>213</v>
+      </c>
+      <c r="H11" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="O11" s="30"/>
+      <c r="O11" s="29"/>
       <c r="U11" s="25" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="H12" s="29" t="s">
+        <v>215</v>
+      </c>
+      <c r="H12" s="28" t="s">
         <v>27</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="O12" s="30"/>
+      <c r="O12" s="29"/>
       <c r="U12" s="25" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="H13" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="H13" s="28" t="s">
         <v>67</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="O13" s="30"/>
+      <c r="O13" s="29"/>
       <c r="U13" s="25" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="H14" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="H14" s="28" t="s">
         <v>67</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="O14" s="30"/>
+      <c r="O14" s="29"/>
       <c r="U14" s="25" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="H15" s="29" t="s">
-        <v>202</v>
+        <v>219</v>
+      </c>
+      <c r="H15" s="28" t="s">
+        <v>207</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="M15" s="30"/>
-      <c r="O15" s="30"/>
+        <v>220</v>
+      </c>
+      <c r="M15" s="29"/>
+      <c r="O15" s="29"/>
       <c r="U15" s="25" t="s">
         <v>135</v>
       </c>
@@ -7911,1237 +7508,257 @@
       <c r="B16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H16" s="29" t="s">
-        <v>202</v>
+      <c r="H16" s="28" t="s">
+        <v>207</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="M16" s="30"/>
+        <v>221</v>
+      </c>
+      <c r="M16" s="29"/>
       <c r="U16" s="25" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H17" s="29" t="s">
+      <c r="H17" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="M17" s="30"/>
-      <c r="U17" s="30"/>
+        <v>222</v>
+      </c>
+      <c r="M17" s="29"/>
+      <c r="U17" s="29"/>
     </row>
     <row r="18" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H18" s="29" t="s">
+      <c r="H18" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M18" s="30"/>
-      <c r="U18" s="30"/>
+      <c r="M18" s="29"/>
+      <c r="U18" s="29"/>
     </row>
     <row r="19" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H19" s="29" t="s">
+      <c r="H19" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="M19" s="30"/>
-      <c r="U19" s="30"/>
+      <c r="M19" s="29"/>
+      <c r="U19" s="29"/>
     </row>
     <row r="20" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H20" s="29" t="s">
+      <c r="H20" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="M20" s="30"/>
-      <c r="U20" s="30"/>
+        <v>223</v>
+      </c>
+      <c r="M20" s="29"/>
+      <c r="U20" s="29"/>
     </row>
     <row r="21" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H21" s="29" t="s">
+      <c r="H21" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="M21" s="30"/>
-      <c r="U21" s="30"/>
+      <c r="M21" s="29"/>
+      <c r="U21" s="29"/>
     </row>
     <row r="22" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H22" s="29" t="s">
+      <c r="H22" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M22" s="30"/>
-      <c r="U22" s="30"/>
+      <c r="M22" s="29"/>
+      <c r="U22" s="29"/>
     </row>
     <row r="23" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H23" s="29" t="s">
+      <c r="H23" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="M23" s="30"/>
-      <c r="U23" s="30"/>
+        <v>224</v>
+      </c>
+      <c r="M23" s="29"/>
+      <c r="U23" s="29"/>
     </row>
     <row r="24" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H24" s="29" t="s">
+      <c r="H24" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="M24" s="30"/>
-      <c r="U24" s="30"/>
+        <v>225</v>
+      </c>
+      <c r="M24" s="29"/>
+      <c r="U24" s="29"/>
     </row>
     <row r="25" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H25" s="29" t="s">
+      <c r="H25" s="28" t="s">
         <v>43</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M25" s="30"/>
-      <c r="U25" s="30"/>
+      <c r="M25" s="29"/>
+      <c r="U25" s="29"/>
     </row>
     <row r="26" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H26" s="29" t="s">
+      <c r="H26" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M26" s="30"/>
-      <c r="U26" s="30"/>
+      <c r="M26" s="29"/>
+      <c r="U26" s="29"/>
     </row>
     <row r="27" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H27" s="29" t="s">
+      <c r="H27" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="M27" s="30"/>
-      <c r="U27" s="30"/>
+      <c r="M27" s="29"/>
+      <c r="U27" s="29"/>
     </row>
     <row r="28" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H28" s="29" t="s">
+      <c r="H28" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="M28" s="30"/>
-      <c r="U28" s="30"/>
+      <c r="M28" s="29"/>
+      <c r="U28" s="29"/>
     </row>
     <row r="29" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H29" s="29" t="s">
+      <c r="H29" s="28" t="s">
         <v>54</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M29" s="30"/>
-      <c r="U29" s="30"/>
+      <c r="M29" s="29"/>
+      <c r="U29" s="29"/>
     </row>
     <row r="30" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H30" s="29" t="s">
+      <c r="H30" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="M30" s="30"/>
-      <c r="U30" s="30"/>
+      <c r="M30" s="29"/>
+      <c r="U30" s="29"/>
     </row>
     <row r="31" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H31" s="29" t="s">
+      <c r="H31" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="M31" s="30"/>
-      <c r="U31" s="30"/>
+      <c r="M31" s="29"/>
+      <c r="U31" s="29"/>
     </row>
     <row r="32" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H32" s="29" t="s">
+      <c r="H32" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="M32" s="30"/>
-      <c r="U32" s="30"/>
+        <v>226</v>
+      </c>
+      <c r="M32" s="29"/>
+      <c r="U32" s="29"/>
     </row>
     <row r="33" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H33" s="29" t="s">
+      <c r="H33" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="M33" s="30"/>
-      <c r="U33" s="30"/>
+        <v>227</v>
+      </c>
+      <c r="M33" s="29"/>
+      <c r="U33" s="29"/>
     </row>
     <row r="34" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H34" s="29" t="s">
+      <c r="H34" s="28" t="s">
         <v>32</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M34" s="30"/>
-      <c r="U34" s="30"/>
+      <c r="M34" s="29"/>
+      <c r="U34" s="29"/>
     </row>
     <row r="35" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H35" s="29" t="s">
-        <v>193</v>
+      <c r="H35" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="M35" s="30"/>
-      <c r="U35" s="30"/>
+        <v>228</v>
+      </c>
+      <c r="M35" s="29"/>
+      <c r="U35" s="29"/>
     </row>
     <row r="36" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H36" s="29" t="s">
-        <v>193</v>
+      <c r="H36" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="M36" s="30"/>
-      <c r="U36" s="30"/>
+        <v>229</v>
+      </c>
+      <c r="M36" s="29"/>
+      <c r="U36" s="29"/>
     </row>
     <row r="37" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H37" s="29" t="s">
-        <v>193</v>
+      <c r="H37" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="M37" s="30"/>
-      <c r="U37" s="30"/>
+        <v>230</v>
+      </c>
+      <c r="M37" s="29"/>
+      <c r="U37" s="29"/>
     </row>
     <row r="38" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H38" s="29" t="s">
-        <v>193</v>
+      <c r="H38" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="M38" s="30"/>
-      <c r="U38" s="30"/>
+        <v>231</v>
+      </c>
+      <c r="M38" s="29"/>
+      <c r="U38" s="29"/>
     </row>
     <row r="39" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H39" s="29" t="s">
-        <v>193</v>
+      <c r="H39" s="28" t="s">
+        <v>198</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="M39" s="30"/>
-      <c r="U39" s="30"/>
-    </row>
-    <row r="40" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M40" s="30"/>
-      <c r="U40" s="30"/>
-    </row>
-    <row r="41" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M41" s="30"/>
-      <c r="U41" s="30"/>
-    </row>
-    <row r="42" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M42" s="30"/>
-      <c r="U42" s="30"/>
-    </row>
-    <row r="43" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M43" s="30"/>
-      <c r="U43" s="30"/>
-    </row>
-    <row r="44" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M44" s="30"/>
-      <c r="U44" s="30"/>
-    </row>
-    <row r="45" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M45" s="30"/>
-      <c r="U45" s="30"/>
-    </row>
-    <row r="46" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M46" s="30"/>
-      <c r="U46" s="30"/>
-    </row>
-    <row r="47" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M47" s="30"/>
-      <c r="U47" s="30"/>
-    </row>
-    <row r="48" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M48" s="30"/>
-      <c r="U48" s="30"/>
-    </row>
-    <row r="49" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M49" s="30"/>
-      <c r="U49" s="30"/>
-    </row>
-    <row r="50" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M50" s="30"/>
-      <c r="U50" s="30"/>
-    </row>
-    <row r="51" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M51" s="30"/>
-      <c r="U51" s="30"/>
-    </row>
-    <row r="52" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M52" s="30"/>
-      <c r="U52" s="30"/>
-    </row>
-    <row r="53" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M53" s="30"/>
-      <c r="U53" s="30"/>
-    </row>
-    <row r="54" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M54" s="30"/>
-      <c r="U54" s="30"/>
-    </row>
-    <row r="55" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M55" s="30"/>
-      <c r="U55" s="30"/>
-    </row>
-    <row r="56" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M56" s="30"/>
-      <c r="U56" s="30"/>
-    </row>
-    <row r="57" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M57" s="30"/>
-      <c r="U57" s="30"/>
-    </row>
-    <row r="58" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M58" s="30"/>
-      <c r="U58" s="30"/>
-    </row>
-    <row r="59" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M59" s="30"/>
-      <c r="U59" s="30"/>
-    </row>
-    <row r="60" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M60" s="30"/>
-      <c r="U60" s="30"/>
-    </row>
-    <row r="61" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M61" s="30"/>
-      <c r="U61" s="30"/>
-    </row>
-    <row r="62" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M62" s="30"/>
-      <c r="U62" s="30"/>
-    </row>
-    <row r="63" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M63" s="30"/>
-      <c r="U63" s="30"/>
-    </row>
-    <row r="64" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M64" s="30"/>
-      <c r="U64" s="30"/>
-    </row>
-    <row r="65" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M65" s="30"/>
-      <c r="U65" s="30"/>
-    </row>
-    <row r="66" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M66" s="30"/>
-      <c r="U66" s="30"/>
-    </row>
-    <row r="67" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M67" s="30"/>
-      <c r="U67" s="30"/>
-    </row>
-    <row r="68" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M68" s="30"/>
-      <c r="U68" s="30"/>
-    </row>
-    <row r="69" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M69" s="30"/>
-      <c r="U69" s="30"/>
-    </row>
-    <row r="70" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M70" s="30"/>
-      <c r="U70" s="30"/>
-    </row>
-    <row r="71" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M71" s="30"/>
-      <c r="U71" s="30"/>
-    </row>
-    <row r="72" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M72" s="30"/>
-      <c r="U72" s="30"/>
-    </row>
-    <row r="73" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M73" s="30"/>
-      <c r="U73" s="30"/>
-    </row>
-    <row r="74" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M74" s="30"/>
-      <c r="U74" s="30"/>
-    </row>
-    <row r="75" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M75" s="30"/>
-      <c r="U75" s="30"/>
-    </row>
-    <row r="76" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M76" s="30"/>
-      <c r="U76" s="30"/>
-    </row>
-    <row r="77" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M77" s="30"/>
-      <c r="U77" s="30"/>
-    </row>
-    <row r="78" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M78" s="30"/>
-      <c r="U78" s="30"/>
-    </row>
-    <row r="79" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M79" s="30"/>
-      <c r="U79" s="30"/>
-    </row>
-    <row r="80" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M80" s="30"/>
-      <c r="U80" s="30"/>
-    </row>
-    <row r="81" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M81" s="30"/>
-      <c r="U81" s="30"/>
-    </row>
-    <row r="82" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M82" s="30"/>
-      <c r="U82" s="30"/>
-    </row>
-    <row r="83" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M83" s="30"/>
-      <c r="U83" s="30"/>
-    </row>
-    <row r="84" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M84" s="30"/>
-      <c r="U84" s="30"/>
-    </row>
-    <row r="85" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M85" s="30"/>
-      <c r="U85" s="30"/>
-    </row>
-    <row r="86" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M86" s="30"/>
-      <c r="U86" s="30"/>
-    </row>
-    <row r="87" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M87" s="30"/>
-      <c r="U87" s="30"/>
-    </row>
-    <row r="88" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M88" s="30"/>
-      <c r="U88" s="30"/>
-    </row>
-    <row r="89" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M89" s="30"/>
-      <c r="U89" s="30"/>
-    </row>
-    <row r="90" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M90" s="30"/>
-      <c r="U90" s="30"/>
-    </row>
-    <row r="91" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M91" s="30"/>
-      <c r="U91" s="30"/>
-    </row>
-    <row r="92" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M92" s="30"/>
-      <c r="U92" s="30"/>
-    </row>
-    <row r="93" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M93" s="30"/>
-      <c r="U93" s="30"/>
-    </row>
-    <row r="94" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M94" s="30"/>
-      <c r="U94" s="30"/>
-    </row>
-    <row r="95" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M95" s="30"/>
-      <c r="U95" s="30"/>
-    </row>
-    <row r="96" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M96" s="30"/>
-      <c r="U96" s="30"/>
-    </row>
-    <row r="97" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M97" s="30"/>
-      <c r="U97" s="30"/>
-    </row>
-    <row r="98" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M98" s="30"/>
-      <c r="U98" s="30"/>
-    </row>
-    <row r="99" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M99" s="30"/>
-      <c r="U99" s="30"/>
-    </row>
-    <row r="100" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M100" s="30"/>
-      <c r="U100" s="30"/>
-    </row>
-    <row r="101" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M101" s="30"/>
-      <c r="U101" s="30"/>
-    </row>
-    <row r="102" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M102" s="30"/>
-      <c r="U102" s="30"/>
-    </row>
-    <row r="103" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M103" s="30"/>
-      <c r="U103" s="30"/>
-    </row>
-    <row r="104" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M104" s="30"/>
-      <c r="U104" s="30"/>
-    </row>
-    <row r="105" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M105" s="30"/>
-      <c r="U105" s="30"/>
-    </row>
-    <row r="106" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M106" s="30"/>
-      <c r="U106" s="30"/>
-    </row>
-    <row r="107" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M107" s="30"/>
-      <c r="U107" s="30"/>
-    </row>
-    <row r="108" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M108" s="30"/>
-      <c r="U108" s="30"/>
-    </row>
-    <row r="109" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M109" s="30"/>
-      <c r="U109" s="30"/>
-    </row>
-    <row r="110" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M110" s="30"/>
-      <c r="U110" s="30"/>
-    </row>
-    <row r="111" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M111" s="30"/>
-      <c r="U111" s="30"/>
-    </row>
-    <row r="112" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M112" s="30"/>
-      <c r="U112" s="30"/>
-    </row>
-    <row r="113" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M113" s="30"/>
-      <c r="U113" s="30"/>
-    </row>
-    <row r="114" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M114" s="30"/>
-      <c r="U114" s="30"/>
-    </row>
-    <row r="115" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M115" s="30"/>
-      <c r="U115" s="30"/>
-    </row>
-    <row r="116" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M116" s="30"/>
-      <c r="U116" s="30"/>
-    </row>
-    <row r="117" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M117" s="30"/>
-      <c r="U117" s="30"/>
-    </row>
-    <row r="118" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M118" s="30"/>
-      <c r="U118" s="30"/>
-    </row>
-    <row r="119" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M119" s="30"/>
-      <c r="U119" s="30"/>
-    </row>
-    <row r="120" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M120" s="30"/>
-      <c r="U120" s="30"/>
-    </row>
-    <row r="121" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M121" s="30"/>
-      <c r="U121" s="30"/>
-    </row>
-    <row r="122" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M122" s="30"/>
-      <c r="U122" s="30"/>
-    </row>
-    <row r="123" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M123" s="30"/>
-      <c r="U123" s="30"/>
-    </row>
-    <row r="124" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M124" s="30"/>
-      <c r="U124" s="30"/>
-    </row>
-    <row r="125" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M125" s="30"/>
-      <c r="U125" s="30"/>
-    </row>
-    <row r="126" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M126" s="30"/>
-      <c r="U126" s="30"/>
-    </row>
-    <row r="127" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M127" s="30"/>
-      <c r="U127" s="30"/>
-    </row>
-    <row r="128" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M128" s="30"/>
-      <c r="U128" s="30"/>
-    </row>
-    <row r="129" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M129" s="30"/>
-      <c r="U129" s="30"/>
-    </row>
-    <row r="130" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M130" s="30"/>
-      <c r="U130" s="30"/>
-    </row>
-    <row r="131" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M131" s="30"/>
-      <c r="U131" s="30"/>
-    </row>
-    <row r="132" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M132" s="30"/>
-      <c r="U132" s="30"/>
-    </row>
-    <row r="133" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M133" s="30"/>
-      <c r="U133" s="30"/>
-    </row>
-    <row r="134" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M134" s="30"/>
-      <c r="U134" s="30"/>
-    </row>
-    <row r="135" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M135" s="30"/>
-      <c r="U135" s="30"/>
-    </row>
-    <row r="136" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M136" s="30"/>
-      <c r="U136" s="30"/>
-    </row>
-    <row r="137" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M137" s="30"/>
-      <c r="U137" s="30"/>
-    </row>
-    <row r="138" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M138" s="30"/>
-      <c r="U138" s="30"/>
-    </row>
-    <row r="139" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M139" s="30"/>
-      <c r="U139" s="30"/>
-    </row>
-    <row r="140" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M140" s="30"/>
-      <c r="U140" s="30"/>
-    </row>
-    <row r="141" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M141" s="30"/>
-      <c r="U141" s="30"/>
-    </row>
-    <row r="142" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M142" s="30"/>
-      <c r="U142" s="30"/>
-    </row>
-    <row r="143" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M143" s="30"/>
-      <c r="U143" s="30"/>
-    </row>
-    <row r="144" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M144" s="30"/>
-      <c r="U144" s="30"/>
-    </row>
-    <row r="145" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M145" s="30"/>
-      <c r="U145" s="30"/>
-    </row>
-    <row r="146" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M146" s="30"/>
-      <c r="U146" s="30"/>
-    </row>
-    <row r="147" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M147" s="30"/>
-      <c r="U147" s="30"/>
-    </row>
-    <row r="148" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M148" s="30"/>
-      <c r="U148" s="30"/>
-    </row>
-    <row r="149" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M149" s="30"/>
-      <c r="U149" s="30"/>
-    </row>
-    <row r="150" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M150" s="30"/>
-    </row>
-    <row r="151" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M151" s="30"/>
-    </row>
-    <row r="152" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M152" s="30"/>
-    </row>
-    <row r="153" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M153" s="30"/>
-    </row>
-    <row r="154" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M154" s="30"/>
-    </row>
-    <row r="155" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M155" s="30"/>
-    </row>
-    <row r="156" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M156" s="30"/>
-    </row>
-    <row r="157" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M157" s="30"/>
-    </row>
-    <row r="158" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M158" s="30"/>
-    </row>
-    <row r="159" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M159" s="30"/>
-    </row>
-    <row r="160" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M160" s="30"/>
-    </row>
-    <row r="161" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M161" s="30"/>
-    </row>
-    <row r="162" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M162" s="30"/>
-    </row>
-    <row r="163" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M163" s="30"/>
-    </row>
-    <row r="164" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M164" s="30"/>
-    </row>
-    <row r="165" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M165" s="30"/>
-    </row>
-    <row r="166" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M166" s="30"/>
-    </row>
-    <row r="167" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M167" s="30"/>
-    </row>
-    <row r="168" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M168" s="30"/>
-    </row>
-    <row r="169" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M169" s="30"/>
-    </row>
-    <row r="170" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M170" s="30"/>
-    </row>
-    <row r="171" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M171" s="30"/>
-    </row>
-    <row r="172" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M172" s="30"/>
-    </row>
-    <row r="173" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M173" s="30"/>
-    </row>
-    <row r="174" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M174" s="30"/>
-    </row>
-    <row r="175" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M175" s="30"/>
-    </row>
-    <row r="176" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M176" s="30"/>
-    </row>
-    <row r="177" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M177" s="30"/>
-    </row>
-    <row r="178" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M178" s="30"/>
-    </row>
-    <row r="179" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M179" s="30"/>
-    </row>
-    <row r="180" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M180" s="30"/>
-    </row>
-    <row r="181" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M181" s="30"/>
-    </row>
-    <row r="182" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M182" s="30"/>
-    </row>
-    <row r="183" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M183" s="30"/>
-    </row>
-    <row r="184" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M184" s="30"/>
-    </row>
-    <row r="185" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M185" s="30"/>
-    </row>
-    <row r="186" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M186" s="30"/>
-    </row>
-    <row r="187" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M187" s="30"/>
-    </row>
-    <row r="188" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M188" s="30"/>
-    </row>
-    <row r="189" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M189" s="30"/>
-    </row>
-    <row r="190" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M190" s="30"/>
-    </row>
-    <row r="191" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M191" s="30"/>
-    </row>
-    <row r="192" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M192" s="30"/>
-    </row>
-    <row r="193" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M193" s="30"/>
-    </row>
-    <row r="194" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M194" s="30"/>
-    </row>
-    <row r="195" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M195" s="30"/>
-    </row>
-    <row r="196" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M196" s="30"/>
-    </row>
-    <row r="197" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M197" s="30"/>
-    </row>
-    <row r="198" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M198" s="30"/>
-    </row>
-    <row r="199" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M199" s="30"/>
-    </row>
-    <row r="200" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M200" s="30"/>
-    </row>
-    <row r="201" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M201" s="30"/>
-    </row>
-    <row r="202" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M202" s="30"/>
-    </row>
-    <row r="203" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M203" s="30"/>
-    </row>
-    <row r="204" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M204" s="30"/>
-    </row>
-    <row r="205" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M205" s="30"/>
-    </row>
-    <row r="206" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M206" s="30"/>
-    </row>
-    <row r="207" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M207" s="30"/>
-    </row>
-    <row r="208" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M208" s="30"/>
-    </row>
-    <row r="209" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M209" s="30"/>
-    </row>
-    <row r="210" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M210" s="30"/>
-    </row>
-    <row r="211" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M211" s="30"/>
-    </row>
-    <row r="212" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M212" s="30"/>
-    </row>
-    <row r="213" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M213" s="30"/>
-    </row>
-    <row r="214" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M214" s="30"/>
-    </row>
-    <row r="215" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M215" s="30"/>
-    </row>
-    <row r="216" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M216" s="30"/>
-    </row>
-    <row r="217" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M217" s="30"/>
-    </row>
-    <row r="218" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M218" s="30"/>
-    </row>
-    <row r="219" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M219" s="30"/>
-    </row>
-    <row r="220" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M220" s="30"/>
-    </row>
-    <row r="221" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M221" s="30"/>
-    </row>
-    <row r="222" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M222" s="30"/>
-    </row>
-    <row r="223" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M223" s="30"/>
-    </row>
-    <row r="224" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M224" s="30"/>
-    </row>
-    <row r="225" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M225" s="30"/>
-    </row>
-    <row r="226" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M226" s="30"/>
-    </row>
-    <row r="227" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M227" s="30"/>
-    </row>
-    <row r="228" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M228" s="30"/>
-    </row>
-    <row r="229" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M229" s="30"/>
-    </row>
-    <row r="230" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M230" s="30"/>
-    </row>
-    <row r="231" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M231" s="30"/>
-    </row>
-    <row r="232" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M232" s="30"/>
-    </row>
-    <row r="233" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M233" s="30"/>
-    </row>
-    <row r="234" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M234" s="30"/>
-    </row>
-    <row r="235" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M235" s="30"/>
-    </row>
-    <row r="236" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M236" s="30"/>
-    </row>
-    <row r="237" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M237" s="30"/>
-    </row>
-    <row r="238" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M238" s="30"/>
-    </row>
-    <row r="239" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M239" s="30"/>
-    </row>
-    <row r="240" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M240" s="30"/>
-    </row>
-    <row r="241" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M241" s="30"/>
-    </row>
-    <row r="242" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M242" s="30"/>
-    </row>
-    <row r="243" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M243" s="30"/>
-    </row>
-    <row r="244" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M244" s="30"/>
-    </row>
-    <row r="245" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M245" s="30"/>
-    </row>
-    <row r="246" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M246" s="30"/>
-    </row>
-    <row r="247" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M247" s="30"/>
-    </row>
-    <row r="248" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M248" s="30"/>
-    </row>
-    <row r="249" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M249" s="30"/>
-    </row>
-    <row r="250" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M250" s="30"/>
-    </row>
-    <row r="251" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M251" s="30"/>
-    </row>
-    <row r="252" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M252" s="30"/>
-    </row>
-    <row r="253" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M253" s="30"/>
-    </row>
-    <row r="254" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M254" s="30"/>
-    </row>
-    <row r="255" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M255" s="30"/>
-    </row>
-    <row r="256" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M256" s="30"/>
-    </row>
-    <row r="257" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M257" s="30"/>
-    </row>
-    <row r="258" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M258" s="30"/>
-    </row>
-    <row r="259" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M259" s="30"/>
-    </row>
-    <row r="260" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M260" s="30"/>
-    </row>
-    <row r="261" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M261" s="30"/>
-    </row>
-    <row r="262" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M262" s="30"/>
-    </row>
-    <row r="263" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M263" s="30"/>
-    </row>
-    <row r="264" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M264" s="30"/>
-    </row>
-    <row r="265" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M265" s="30"/>
-    </row>
-    <row r="266" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M266" s="30"/>
-    </row>
-    <row r="267" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M267" s="30"/>
-    </row>
-    <row r="268" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M268" s="30"/>
-    </row>
-    <row r="269" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M269" s="30"/>
-    </row>
-    <row r="270" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M270" s="30"/>
-    </row>
-    <row r="271" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M271" s="30"/>
-    </row>
-    <row r="272" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M272" s="30"/>
-    </row>
-    <row r="273" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M273" s="30"/>
-    </row>
-    <row r="274" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M274" s="30"/>
-    </row>
-    <row r="275" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M275" s="30"/>
-    </row>
-    <row r="276" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M276" s="30"/>
-    </row>
-    <row r="277" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M277" s="30"/>
-    </row>
-    <row r="278" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M278" s="30"/>
-    </row>
-    <row r="279" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M279" s="30"/>
-    </row>
-    <row r="280" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M280" s="30"/>
-    </row>
-    <row r="281" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M281" s="30"/>
-    </row>
-    <row r="282" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M282" s="30"/>
-    </row>
-    <row r="283" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M283" s="30"/>
-    </row>
-    <row r="284" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M284" s="30"/>
-    </row>
-    <row r="285" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M285" s="30"/>
-    </row>
-    <row r="286" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M286" s="30"/>
-    </row>
-    <row r="287" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M287" s="30"/>
-    </row>
-    <row r="288" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M288" s="30"/>
-    </row>
-    <row r="289" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M289" s="30"/>
-    </row>
-    <row r="290" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M290" s="30"/>
-    </row>
-    <row r="291" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M291" s="30"/>
-    </row>
-    <row r="292" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M292" s="30"/>
-    </row>
-    <row r="293" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M293" s="30"/>
-    </row>
-    <row r="294" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M294" s="30"/>
-    </row>
-    <row r="295" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M295" s="30"/>
-    </row>
-    <row r="296" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M296" s="30"/>
-    </row>
-    <row r="297" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M297" s="30"/>
-    </row>
-    <row r="298" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M298" s="30"/>
-    </row>
-    <row r="299" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M299" s="30"/>
-    </row>
-    <row r="300" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M300" s="30"/>
-    </row>
-    <row r="301" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M301" s="30"/>
-    </row>
-    <row r="302" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M302" s="30"/>
-    </row>
-    <row r="303" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M303" s="30"/>
-    </row>
-    <row r="304" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M304" s="30"/>
-    </row>
-    <row r="305" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M305" s="30"/>
-    </row>
-    <row r="306" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M306" s="30"/>
-    </row>
-    <row r="307" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M307" s="30"/>
-    </row>
-    <row r="308" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M308" s="30"/>
-    </row>
-    <row r="309" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M309" s="30"/>
-    </row>
-    <row r="310" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M310" s="30"/>
-    </row>
-    <row r="311" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M311" s="30"/>
-    </row>
-    <row r="312" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M312" s="30"/>
-    </row>
-    <row r="313" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M313" s="30"/>
-    </row>
-    <row r="314" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M314" s="30"/>
-    </row>
-    <row r="315" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M315" s="30"/>
-    </row>
-    <row r="316" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M316" s="30"/>
-    </row>
-    <row r="317" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M317" s="30"/>
-    </row>
-    <row r="318" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M318" s="30"/>
-    </row>
-    <row r="319" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M319" s="30"/>
-    </row>
-    <row r="320" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M320" s="30"/>
-    </row>
-    <row r="321" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M321" s="30"/>
-    </row>
-    <row r="322" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M322" s="30"/>
-    </row>
-    <row r="323" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M323" s="30"/>
-    </row>
-    <row r="324" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M324" s="30"/>
-    </row>
-    <row r="325" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M325" s="30"/>
-    </row>
-    <row r="326" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M326" s="30"/>
-    </row>
-    <row r="327" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M327" s="30"/>
-    </row>
-    <row r="328" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M328" s="30"/>
-    </row>
-    <row r="329" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M329" s="30"/>
+      <c r="M39" s="29"/>
+      <c r="U39" s="29"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H3:H39" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="H3:H39" type="list">
       <formula1>$K$3:$K$9</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9158,15 +7775,15 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="2.99"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="2"/>
   </cols>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9183,8 +7800,8 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>